<commit_message>
Fixing mismatch between metric file variable names and name_matching.R and creating a check for if there are missing variables not included in dataframe
</commit_message>
<xml_diff>
--- a/data/1_production_model/static_tables/metric_structure.xlsx
+++ b/data/1_production_model/static_tables/metric_structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\static_tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\zhangm\egrid-git\data\1_production_model\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BB9FB4-03D0-4599-A2C0-AD596F345934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579E1706-064D-46AB-8613-0B1EDF89F43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5490" yWindow="1590" windowWidth="23310" windowHeight="14010" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unit_annual" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12212" uniqueCount="4566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12212" uniqueCount="4561">
   <si>
     <t>Name</t>
   </si>
@@ -12687,102 +12687,6 @@
     <t>PLGENMCO2</t>
   </si>
   <si>
-    <t>STHTIMO</t>
-  </si>
-  <si>
-    <t>STHTIMOT</t>
-  </si>
-  <si>
-    <t>STNGENMO</t>
-  </si>
-  <si>
-    <t>STNGENMO2</t>
-  </si>
-  <si>
-    <t>STNOXMO</t>
-  </si>
-  <si>
-    <t>STSO2MO</t>
-  </si>
-  <si>
-    <t>STCO2MO</t>
-  </si>
-  <si>
-    <t>STCH4MO</t>
-  </si>
-  <si>
-    <t>STN2OMO</t>
-  </si>
-  <si>
-    <t>STHGMO</t>
-  </si>
-  <si>
-    <t>STCO2EQM</t>
-  </si>
-  <si>
-    <t>STNOXRTM</t>
-  </si>
-  <si>
-    <t>STNOXRTM2</t>
-  </si>
-  <si>
-    <t>STSO2RTM</t>
-  </si>
-  <si>
-    <t>STSO2RTM2</t>
-  </si>
-  <si>
-    <t>STCO2RTM</t>
-  </si>
-  <si>
-    <t>STCO2RTM2</t>
-  </si>
-  <si>
-    <t>STCH4RTM</t>
-  </si>
-  <si>
-    <t>STCH4RTM2</t>
-  </si>
-  <si>
-    <t>STN2ORTM</t>
-  </si>
-  <si>
-    <t>STN2ORTM2</t>
-  </si>
-  <si>
-    <t>STC2ERTM</t>
-  </si>
-  <si>
-    <t>STC2ERTM2</t>
-  </si>
-  <si>
-    <t>STHGRTM</t>
-  </si>
-  <si>
-    <t>STHGRTM2</t>
-  </si>
-  <si>
-    <t>STNOXRM</t>
-  </si>
-  <si>
-    <t>STSO2RM</t>
-  </si>
-  <si>
-    <t>STCO2RM</t>
-  </si>
-  <si>
-    <t>STCH4RM</t>
-  </si>
-  <si>
-    <t>STN2ORM</t>
-  </si>
-  <si>
-    <t>STC2ERM</t>
-  </si>
-  <si>
-    <t>STHGRM</t>
-  </si>
-  <si>
     <t>STGENMCL</t>
   </si>
   <si>
@@ -12891,102 +12795,6 @@
     <t>STGENMCO2</t>
   </si>
   <si>
-    <t>BAHTIMO</t>
-  </si>
-  <si>
-    <t>BAHTIMOT</t>
-  </si>
-  <si>
-    <t>BANGENMO</t>
-  </si>
-  <si>
-    <t>BANGENMO2</t>
-  </si>
-  <si>
-    <t>BANOXMO</t>
-  </si>
-  <si>
-    <t>BASO2MO</t>
-  </si>
-  <si>
-    <t>BACO2MO</t>
-  </si>
-  <si>
-    <t>BACH4MO</t>
-  </si>
-  <si>
-    <t>BAN2OMO</t>
-  </si>
-  <si>
-    <t>BACO2EQM</t>
-  </si>
-  <si>
-    <t>BAHGMO</t>
-  </si>
-  <si>
-    <t>BANOXRTM</t>
-  </si>
-  <si>
-    <t>BANOXRTM2</t>
-  </si>
-  <si>
-    <t>BASO2RTM</t>
-  </si>
-  <si>
-    <t>BASO2RTM2</t>
-  </si>
-  <si>
-    <t>BACO2RTM</t>
-  </si>
-  <si>
-    <t>BACO2RTM2</t>
-  </si>
-  <si>
-    <t>BACH4RTM</t>
-  </si>
-  <si>
-    <t>BACH4RTM2</t>
-  </si>
-  <si>
-    <t>BAN2ORTM</t>
-  </si>
-  <si>
-    <t>BAN2ORTM2</t>
-  </si>
-  <si>
-    <t>BAC2ERTM</t>
-  </si>
-  <si>
-    <t>BAC2ERTM2</t>
-  </si>
-  <si>
-    <t>BAHGRTM</t>
-  </si>
-  <si>
-    <t>BAHGRTM2</t>
-  </si>
-  <si>
-    <t>BANOXRM</t>
-  </si>
-  <si>
-    <t>BASO2RM</t>
-  </si>
-  <si>
-    <t>BACO2RM</t>
-  </si>
-  <si>
-    <t>BACH4RM</t>
-  </si>
-  <si>
-    <t>BAN2ORM</t>
-  </si>
-  <si>
-    <t>BAC2ERM</t>
-  </si>
-  <si>
-    <t>BAHGRM</t>
-  </si>
-  <si>
     <t>BAGENMCL</t>
   </si>
   <si>
@@ -13092,102 +12900,6 @@
     <t>BAGENMCO2</t>
   </si>
   <si>
-    <t>SRNOXMO</t>
-  </si>
-  <si>
-    <t>SRHTIMO</t>
-  </si>
-  <si>
-    <t>SRHTIMOT</t>
-  </si>
-  <si>
-    <t>SRNGENMO</t>
-  </si>
-  <si>
-    <t>SRNGENMO2</t>
-  </si>
-  <si>
-    <t>SRSO2MO</t>
-  </si>
-  <si>
-    <t>SRCO2MO</t>
-  </si>
-  <si>
-    <t>SRCH4MO</t>
-  </si>
-  <si>
-    <t>SRN2OMO</t>
-  </si>
-  <si>
-    <t>SRCO2EQM</t>
-  </si>
-  <si>
-    <t>SRHGMO</t>
-  </si>
-  <si>
-    <t>SRNOXRTM</t>
-  </si>
-  <si>
-    <t>SRNOXRTM2</t>
-  </si>
-  <si>
-    <t>SRSO2RTM</t>
-  </si>
-  <si>
-    <t>SRSO2RTM2</t>
-  </si>
-  <si>
-    <t>SRCO2RTM</t>
-  </si>
-  <si>
-    <t>SRCO2RTM2</t>
-  </si>
-  <si>
-    <t>SRCH4RTM</t>
-  </si>
-  <si>
-    <t>SRCH4RTM2</t>
-  </si>
-  <si>
-    <t>SRN2ORTM</t>
-  </si>
-  <si>
-    <t>SRN2ORTM2</t>
-  </si>
-  <si>
-    <t>SRC2ERTM</t>
-  </si>
-  <si>
-    <t>SRC2ERTM2</t>
-  </si>
-  <si>
-    <t>SRHGRTM</t>
-  </si>
-  <si>
-    <t>SRHGRTM2</t>
-  </si>
-  <si>
-    <t>SRNOXRM</t>
-  </si>
-  <si>
-    <t>SRSO2RM</t>
-  </si>
-  <si>
-    <t>SRCO2RM</t>
-  </si>
-  <si>
-    <t>SRCH4RM</t>
-  </si>
-  <si>
-    <t>SRN2ORM</t>
-  </si>
-  <si>
-    <t>SRC2ERM</t>
-  </si>
-  <si>
-    <t>SRHGRM</t>
-  </si>
-  <si>
     <t>SRGENMCL</t>
   </si>
   <si>
@@ -13314,102 +13026,6 @@
     <t>SRNBC2E2</t>
   </si>
   <si>
-    <t>NRHTIMO</t>
-  </si>
-  <si>
-    <t>NRHTIMOT</t>
-  </si>
-  <si>
-    <t>NRNGENMO</t>
-  </si>
-  <si>
-    <t>NRNGENMO2</t>
-  </si>
-  <si>
-    <t>NRNOXMO</t>
-  </si>
-  <si>
-    <t>NRSO2MO</t>
-  </si>
-  <si>
-    <t>NRCO2MO</t>
-  </si>
-  <si>
-    <t>NRCH4MO</t>
-  </si>
-  <si>
-    <t>NRN2OMO</t>
-  </si>
-  <si>
-    <t>NRCO2EQM</t>
-  </si>
-  <si>
-    <t>NRHGMO</t>
-  </si>
-  <si>
-    <t>NRNOXRTM</t>
-  </si>
-  <si>
-    <t>NRNOXRTM2</t>
-  </si>
-  <si>
-    <t>NRSO2RTM</t>
-  </si>
-  <si>
-    <t>NRSO2RTM2</t>
-  </si>
-  <si>
-    <t>NRCO2RTM</t>
-  </si>
-  <si>
-    <t>NRCO2RTM2</t>
-  </si>
-  <si>
-    <t>NRCH4RTM</t>
-  </si>
-  <si>
-    <t>NRCH4RTM2</t>
-  </si>
-  <si>
-    <t>NRN2ORTM</t>
-  </si>
-  <si>
-    <t>NRN2ORTM2</t>
-  </si>
-  <si>
-    <t>NRC2ERTM</t>
-  </si>
-  <si>
-    <t>NRC2ERTM2</t>
-  </si>
-  <si>
-    <t>NRHGRTM</t>
-  </si>
-  <si>
-    <t>NRHGRTM2</t>
-  </si>
-  <si>
-    <t>NRNOXRM</t>
-  </si>
-  <si>
-    <t>NRSO2RM</t>
-  </si>
-  <si>
-    <t>NRCO2RM</t>
-  </si>
-  <si>
-    <t>NRCH4RM</t>
-  </si>
-  <si>
-    <t>NRN2ORM</t>
-  </si>
-  <si>
-    <t>NRC2ERM</t>
-  </si>
-  <si>
-    <t>NRHGRM</t>
-  </si>
-  <si>
     <t>NRGENMCL</t>
   </si>
   <si>
@@ -13518,102 +13134,6 @@
     <t>NRGENMCO2</t>
   </si>
   <si>
-    <t>USHTIMO</t>
-  </si>
-  <si>
-    <t>USHTIMOT</t>
-  </si>
-  <si>
-    <t>USNGENMO</t>
-  </si>
-  <si>
-    <t>USNGENMO2</t>
-  </si>
-  <si>
-    <t>USNOXMO</t>
-  </si>
-  <si>
-    <t>USSO2MO</t>
-  </si>
-  <si>
-    <t>USCO2MO</t>
-  </si>
-  <si>
-    <t>USCH4MO</t>
-  </si>
-  <si>
-    <t>USN2OMO</t>
-  </si>
-  <si>
-    <t>USCO2EQM</t>
-  </si>
-  <si>
-    <t>USHGMO</t>
-  </si>
-  <si>
-    <t>USNOXRTM</t>
-  </si>
-  <si>
-    <t>USNOXRTM2</t>
-  </si>
-  <si>
-    <t>USSO2RTM</t>
-  </si>
-  <si>
-    <t>USSO2RTM2</t>
-  </si>
-  <si>
-    <t>USCO2RTM</t>
-  </si>
-  <si>
-    <t>USCO2RTM2</t>
-  </si>
-  <si>
-    <t>USCH4RTM</t>
-  </si>
-  <si>
-    <t>USCH4RTM2</t>
-  </si>
-  <si>
-    <t>USN2ORTM</t>
-  </si>
-  <si>
-    <t>USN2ORTM2</t>
-  </si>
-  <si>
-    <t>USC2ERTM</t>
-  </si>
-  <si>
-    <t>USC2ERTM2</t>
-  </si>
-  <si>
-    <t>USHGRTM</t>
-  </si>
-  <si>
-    <t>USHGRTM2</t>
-  </si>
-  <si>
-    <t>USNOXRM</t>
-  </si>
-  <si>
-    <t>USSO2RM</t>
-  </si>
-  <si>
-    <t>USCO2RM</t>
-  </si>
-  <si>
-    <t>USCH4RM</t>
-  </si>
-  <si>
-    <t>USN2ORM</t>
-  </si>
-  <si>
-    <t>USC2ERM</t>
-  </si>
-  <si>
-    <t>USHGRM</t>
-  </si>
-  <si>
     <t>USGENMCL</t>
   </si>
   <si>
@@ -13753,6 +13273,471 @@
   </si>
   <si>
     <t>USFSHGRT2</t>
+  </si>
+  <si>
+    <t>STHTIT</t>
+  </si>
+  <si>
+    <t>STNGEN</t>
+  </si>
+  <si>
+    <t>STNGEN2</t>
+  </si>
+  <si>
+    <t>STNOX</t>
+  </si>
+  <si>
+    <t>STSO2</t>
+  </si>
+  <si>
+    <t>STCO2</t>
+  </si>
+  <si>
+    <t>STCH4</t>
+  </si>
+  <si>
+    <t>STN2O</t>
+  </si>
+  <si>
+    <t>STHG</t>
+  </si>
+  <si>
+    <t>STNOXRT</t>
+  </si>
+  <si>
+    <t>STNOXRT2</t>
+  </si>
+  <si>
+    <t>STSO2RT</t>
+  </si>
+  <si>
+    <t>STSO2RT2</t>
+  </si>
+  <si>
+    <t>STCO2RT</t>
+  </si>
+  <si>
+    <t>STCO2RT2</t>
+  </si>
+  <si>
+    <t>STCH4RT</t>
+  </si>
+  <si>
+    <t>STCH4RT2</t>
+  </si>
+  <si>
+    <t>STN2ORT</t>
+  </si>
+  <si>
+    <t>STN2ORT2</t>
+  </si>
+  <si>
+    <t>STC2ERT</t>
+  </si>
+  <si>
+    <t>STC2ERT2</t>
+  </si>
+  <si>
+    <t>STHGRT</t>
+  </si>
+  <si>
+    <t>STNOXR</t>
+  </si>
+  <si>
+    <t>STSO2R</t>
+  </si>
+  <si>
+    <t>STCO2R</t>
+  </si>
+  <si>
+    <t>STCH4R</t>
+  </si>
+  <si>
+    <t>STN2OR</t>
+  </si>
+  <si>
+    <t>STC2ER</t>
+  </si>
+  <si>
+    <t>STHGR</t>
+  </si>
+  <si>
+    <t>BAHTI</t>
+  </si>
+  <si>
+    <t>BAHTIT</t>
+  </si>
+  <si>
+    <t>BANGEN</t>
+  </si>
+  <si>
+    <t>BANGEN2</t>
+  </si>
+  <si>
+    <t>BANOX</t>
+  </si>
+  <si>
+    <t>BASO2</t>
+  </si>
+  <si>
+    <t>BACO2</t>
+  </si>
+  <si>
+    <t>BACH4</t>
+  </si>
+  <si>
+    <t>BAN2O</t>
+  </si>
+  <si>
+    <t>BAHG</t>
+  </si>
+  <si>
+    <t>BANOXRT</t>
+  </si>
+  <si>
+    <t>BANOXRT2</t>
+  </si>
+  <si>
+    <t>BASO2RT</t>
+  </si>
+  <si>
+    <t>BASO2RT2</t>
+  </si>
+  <si>
+    <t>STHTI</t>
+  </si>
+  <si>
+    <t>BACO2RT</t>
+  </si>
+  <si>
+    <t>BACO2RT2</t>
+  </si>
+  <si>
+    <t>BACH4RT</t>
+  </si>
+  <si>
+    <t>BACH4RT2</t>
+  </si>
+  <si>
+    <t>BAN2ORT</t>
+  </si>
+  <si>
+    <t>BAN2ORT2</t>
+  </si>
+  <si>
+    <t>BAC2ERT</t>
+  </si>
+  <si>
+    <t>BAC2ERT2</t>
+  </si>
+  <si>
+    <t>BAHGRT</t>
+  </si>
+  <si>
+    <t>BANOXR</t>
+  </si>
+  <si>
+    <t>BASO2R</t>
+  </si>
+  <si>
+    <t>BACO2R</t>
+  </si>
+  <si>
+    <t>BACH4R</t>
+  </si>
+  <si>
+    <t>BAN2OR</t>
+  </si>
+  <si>
+    <t>BAC2ER</t>
+  </si>
+  <si>
+    <t>BAHGR</t>
+  </si>
+  <si>
+    <t>SRHTI</t>
+  </si>
+  <si>
+    <t>SRHTIT</t>
+  </si>
+  <si>
+    <t>SRNGEN</t>
+  </si>
+  <si>
+    <t>SRNGEN2</t>
+  </si>
+  <si>
+    <t>SRNOX</t>
+  </si>
+  <si>
+    <t>SRSO2</t>
+  </si>
+  <si>
+    <t>SRCO2</t>
+  </si>
+  <si>
+    <t>SRCH4</t>
+  </si>
+  <si>
+    <t>SRN2O</t>
+  </si>
+  <si>
+    <t>SRCO2EQ</t>
+  </si>
+  <si>
+    <t>SRNOXRT</t>
+  </si>
+  <si>
+    <t>SRNOXRT2</t>
+  </si>
+  <si>
+    <t>SRSO2RT</t>
+  </si>
+  <si>
+    <t>SRSO2RT2</t>
+  </si>
+  <si>
+    <t>SRCO2RT</t>
+  </si>
+  <si>
+    <t>SRCO2RT2</t>
+  </si>
+  <si>
+    <t>SRCH4RT</t>
+  </si>
+  <si>
+    <t>SRCH4RT2</t>
+  </si>
+  <si>
+    <t>SRN2ORT</t>
+  </si>
+  <si>
+    <t>SRN2ORT2</t>
+  </si>
+  <si>
+    <t>SRC2ERT</t>
+  </si>
+  <si>
+    <t>SRC2ERT2</t>
+  </si>
+  <si>
+    <t>SRHGRT</t>
+  </si>
+  <si>
+    <t>SRNOXR</t>
+  </si>
+  <si>
+    <t>SRSO2R</t>
+  </si>
+  <si>
+    <t>SRCO2R</t>
+  </si>
+  <si>
+    <t>SRCH4R</t>
+  </si>
+  <si>
+    <t>SRN2OR</t>
+  </si>
+  <si>
+    <t>SRC2ER</t>
+  </si>
+  <si>
+    <t>SRHGR</t>
+  </si>
+  <si>
+    <t>BACO2EQ</t>
+  </si>
+  <si>
+    <t>STCO2EQ</t>
+  </si>
+  <si>
+    <t>SRHG</t>
+  </si>
+  <si>
+    <t>NRHTI</t>
+  </si>
+  <si>
+    <t>NRHTIT</t>
+  </si>
+  <si>
+    <t>NRNGEN</t>
+  </si>
+  <si>
+    <t>NRNGEN2</t>
+  </si>
+  <si>
+    <t>NRNOX</t>
+  </si>
+  <si>
+    <t>NRSO2</t>
+  </si>
+  <si>
+    <t>NRCO2</t>
+  </si>
+  <si>
+    <t>NRCH4</t>
+  </si>
+  <si>
+    <t>NRN2O</t>
+  </si>
+  <si>
+    <t>NRCO2EQ</t>
+  </si>
+  <si>
+    <t>NRHG</t>
+  </si>
+  <si>
+    <t>NRNOXRT</t>
+  </si>
+  <si>
+    <t>NRNOXRT2</t>
+  </si>
+  <si>
+    <t>NRSO2RT</t>
+  </si>
+  <si>
+    <t>NRSO2RT2</t>
+  </si>
+  <si>
+    <t>NRCO2RT</t>
+  </si>
+  <si>
+    <t>NRCO2RT2</t>
+  </si>
+  <si>
+    <t>NRCH4RT</t>
+  </si>
+  <si>
+    <t>NRCH4RT2</t>
+  </si>
+  <si>
+    <t>NRN2ORT</t>
+  </si>
+  <si>
+    <t>NRN2ORT2</t>
+  </si>
+  <si>
+    <t>NRC2ERT</t>
+  </si>
+  <si>
+    <t>NRC2ERT2</t>
+  </si>
+  <si>
+    <t>NRHGRT</t>
+  </si>
+  <si>
+    <t>NRNOXR</t>
+  </si>
+  <si>
+    <t>NRSO2R</t>
+  </si>
+  <si>
+    <t>NRCO2R</t>
+  </si>
+  <si>
+    <t>NRCH4R</t>
+  </si>
+  <si>
+    <t>NRN2OR</t>
+  </si>
+  <si>
+    <t>NRC2ER</t>
+  </si>
+  <si>
+    <t>NRHGR</t>
+  </si>
+  <si>
+    <t>USHTI</t>
+  </si>
+  <si>
+    <t>USHTIT</t>
+  </si>
+  <si>
+    <t>USNGEN</t>
+  </si>
+  <si>
+    <t>USNGEN2</t>
+  </si>
+  <si>
+    <t>USNOX</t>
+  </si>
+  <si>
+    <t>USSO2</t>
+  </si>
+  <si>
+    <t>USCO2</t>
+  </si>
+  <si>
+    <t>USCH4</t>
+  </si>
+  <si>
+    <t>USN2O</t>
+  </si>
+  <si>
+    <t>USCO2EQ</t>
+  </si>
+  <si>
+    <t>USHG</t>
+  </si>
+  <si>
+    <t>USNOXRT</t>
+  </si>
+  <si>
+    <t>USNOXRT2</t>
+  </si>
+  <si>
+    <t>USSO2RT</t>
+  </si>
+  <si>
+    <t>USSO2RT2</t>
+  </si>
+  <si>
+    <t>USCO2RT</t>
+  </si>
+  <si>
+    <t>USCO2RT2</t>
+  </si>
+  <si>
+    <t>USCH4RT</t>
+  </si>
+  <si>
+    <t>USCH4RT2</t>
+  </si>
+  <si>
+    <t>USN2ORT</t>
+  </si>
+  <si>
+    <t>USN2ORT2</t>
+  </si>
+  <si>
+    <t>USC2ERT</t>
+  </si>
+  <si>
+    <t>USC2ERT2</t>
+  </si>
+  <si>
+    <t>USHGRT</t>
+  </si>
+  <si>
+    <t>USNOXR</t>
+  </si>
+  <si>
+    <t>USSO2R</t>
+  </si>
+  <si>
+    <t>USCO2R</t>
+  </si>
+  <si>
+    <t>USCH4R</t>
+  </si>
+  <si>
+    <t>USN2OR</t>
+  </si>
+  <si>
+    <t>USC2ER</t>
+  </si>
+  <si>
+    <t>USHGR</t>
   </si>
 </sst>
 </file>
@@ -15272,7 +15257,7 @@
         <v>3336</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>4278</v>
+        <v>4435</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>31</v>
@@ -15287,7 +15272,7 @@
         <v>3337</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>4279</v>
+        <v>4436</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>31</v>
@@ -15302,7 +15287,7 @@
         <v>3338</v>
       </c>
       <c r="B9" s="52" t="s">
-        <v>4280</v>
+        <v>4437</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>89</v>
@@ -15317,7 +15302,7 @@
         <v>3339</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>4281</v>
+        <v>4438</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>31</v>
@@ -15334,7 +15319,7 @@
         <v>3340</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>4415</v>
+        <v>4319</v>
       </c>
       <c r="C11" s="52" t="s">
         <v>89</v>
@@ -15349,7 +15334,7 @@
         <v>3341</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>4416</v>
+        <v>4320</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>31</v>
@@ -15366,7 +15351,7 @@
         <v>3342</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>4282</v>
+        <v>4439</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>37</v>
@@ -15381,7 +15366,7 @@
         <v>3343</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>4283</v>
+        <v>4440</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>37</v>
@@ -15396,7 +15381,7 @@
         <v>3344</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>4284</v>
+        <v>4441</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>37</v>
@@ -15411,7 +15396,7 @@
         <v>3345</v>
       </c>
       <c r="B16" s="52" t="s">
-        <v>4285</v>
+        <v>4442</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>47</v>
@@ -15426,7 +15411,7 @@
         <v>3346</v>
       </c>
       <c r="B17" s="52" t="s">
-        <v>4286</v>
+        <v>4443</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>47</v>
@@ -15441,7 +15426,7 @@
         <v>3347</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>4287</v>
+        <v>4496</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>37</v>
@@ -15456,7 +15441,7 @@
         <v>3348</v>
       </c>
       <c r="B19" s="52" t="s">
-        <v>4288</v>
+        <v>4444</v>
       </c>
       <c r="C19" s="52" t="s">
         <v>47</v>
@@ -15471,7 +15456,7 @@
         <v>3349</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>4289</v>
+        <v>4445</v>
       </c>
       <c r="C20" s="122" t="s">
         <v>197</v>
@@ -15486,7 +15471,7 @@
         <v>3350</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>4290</v>
+        <v>4446</v>
       </c>
       <c r="C21" s="122" t="s">
         <v>201</v>
@@ -15503,7 +15488,7 @@
         <v>3351</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>4291</v>
+        <v>4447</v>
       </c>
       <c r="C22" s="122" t="s">
         <v>197</v>
@@ -15518,7 +15503,7 @@
         <v>3352</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>4292</v>
+        <v>4448</v>
       </c>
       <c r="C23" s="122" t="s">
         <v>201</v>
@@ -15535,7 +15520,7 @@
         <v>3353</v>
       </c>
       <c r="B24" s="60" t="s">
-        <v>4293</v>
+        <v>4450</v>
       </c>
       <c r="C24" s="122" t="s">
         <v>197</v>
@@ -15550,7 +15535,7 @@
         <v>3354</v>
       </c>
       <c r="B25" s="60" t="s">
-        <v>4294</v>
+        <v>4451</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>201</v>
@@ -15567,7 +15552,7 @@
         <v>3355</v>
       </c>
       <c r="B26" s="60" t="s">
-        <v>4295</v>
+        <v>4452</v>
       </c>
       <c r="C26" s="122" t="s">
         <v>197</v>
@@ -15582,7 +15567,7 @@
         <v>3356</v>
       </c>
       <c r="B27" s="60" t="s">
-        <v>4296</v>
+        <v>4453</v>
       </c>
       <c r="C27" s="122" t="s">
         <v>201</v>
@@ -15599,7 +15584,7 @@
         <v>3357</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>4297</v>
+        <v>4454</v>
       </c>
       <c r="C28" s="122" t="s">
         <v>197</v>
@@ -15614,7 +15599,7 @@
         <v>3358</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>4298</v>
+        <v>4455</v>
       </c>
       <c r="C29" s="122" t="s">
         <v>201</v>
@@ -15631,7 +15616,7 @@
         <v>3359</v>
       </c>
       <c r="B30" s="60" t="s">
-        <v>4299</v>
+        <v>4456</v>
       </c>
       <c r="C30" s="122" t="s">
         <v>197</v>
@@ -15646,7 +15631,7 @@
         <v>3360</v>
       </c>
       <c r="B31" s="60" t="s">
-        <v>4300</v>
+        <v>4457</v>
       </c>
       <c r="C31" s="122" t="s">
         <v>201</v>
@@ -15663,7 +15648,7 @@
         <v>3361</v>
       </c>
       <c r="B32" s="60" t="s">
-        <v>4301</v>
+        <v>4458</v>
       </c>
       <c r="C32" s="122" t="s">
         <v>197</v>
@@ -15678,7 +15663,7 @@
         <v>3362</v>
       </c>
       <c r="B33" s="60" t="s">
-        <v>4302</v>
+        <v>1159</v>
       </c>
       <c r="C33" s="122" t="s">
         <v>201</v>
@@ -15695,7 +15680,7 @@
         <v>3363</v>
       </c>
       <c r="B34" s="62" t="s">
-        <v>4303</v>
+        <v>4459</v>
       </c>
       <c r="C34" s="123" t="s">
         <v>201</v>
@@ -15710,7 +15695,7 @@
         <v>3364</v>
       </c>
       <c r="B35" s="62" t="s">
-        <v>4304</v>
+        <v>4460</v>
       </c>
       <c r="C35" s="123" t="s">
         <v>201</v>
@@ -15725,7 +15710,7 @@
         <v>3365</v>
       </c>
       <c r="B36" s="62" t="s">
-        <v>4305</v>
+        <v>4461</v>
       </c>
       <c r="C36" s="123" t="s">
         <v>201</v>
@@ -15740,7 +15725,7 @@
         <v>3366</v>
       </c>
       <c r="B37" s="62" t="s">
-        <v>4306</v>
+        <v>4462</v>
       </c>
       <c r="C37" s="123" t="s">
         <v>201</v>
@@ -15755,7 +15740,7 @@
         <v>3367</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>4307</v>
+        <v>4463</v>
       </c>
       <c r="C38" s="123" t="s">
         <v>201</v>
@@ -15770,7 +15755,7 @@
         <v>3368</v>
       </c>
       <c r="B39" s="62" t="s">
-        <v>4308</v>
+        <v>4464</v>
       </c>
       <c r="C39" s="123" t="s">
         <v>201</v>
@@ -15785,7 +15770,7 @@
         <v>3369</v>
       </c>
       <c r="B40" s="62" t="s">
-        <v>4309</v>
+        <v>4465</v>
       </c>
       <c r="C40" s="123" t="s">
         <v>201</v>
@@ -16807,7 +16792,7 @@
         <v>3433</v>
       </c>
       <c r="B104" s="96" t="s">
-        <v>1159</v>
+        <v>4399</v>
       </c>
       <c r="C104" s="130" t="s">
         <v>201</v>
@@ -17470,7 +17455,7 @@
         <v>3476</v>
       </c>
       <c r="B147" s="70" t="s">
-        <v>4310</v>
+        <v>4246</v>
       </c>
       <c r="C147" s="70" t="s">
         <v>89</v>
@@ -17485,7 +17470,7 @@
         <v>3477</v>
       </c>
       <c r="B148" s="70" t="s">
-        <v>4311</v>
+        <v>4247</v>
       </c>
       <c r="C148" s="70" t="s">
         <v>31</v>
@@ -17502,7 +17487,7 @@
         <v>3478</v>
       </c>
       <c r="B149" s="70" t="s">
-        <v>4312</v>
+        <v>4248</v>
       </c>
       <c r="C149" s="70" t="s">
         <v>89</v>
@@ -17517,7 +17502,7 @@
         <v>3479</v>
       </c>
       <c r="B150" s="70" t="s">
-        <v>4313</v>
+        <v>4249</v>
       </c>
       <c r="C150" s="70" t="s">
         <v>31</v>
@@ -17534,7 +17519,7 @@
         <v>3480</v>
       </c>
       <c r="B151" s="70" t="s">
-        <v>4314</v>
+        <v>4250</v>
       </c>
       <c r="C151" s="70" t="s">
         <v>89</v>
@@ -17549,7 +17534,7 @@
         <v>3481</v>
       </c>
       <c r="B152" s="70" t="s">
-        <v>4315</v>
+        <v>4251</v>
       </c>
       <c r="C152" s="70" t="s">
         <v>31</v>
@@ -17566,7 +17551,7 @@
         <v>3482</v>
       </c>
       <c r="B153" s="70" t="s">
-        <v>4316</v>
+        <v>4252</v>
       </c>
       <c r="C153" s="70" t="s">
         <v>89</v>
@@ -17581,7 +17566,7 @@
         <v>3483</v>
       </c>
       <c r="B154" s="70" t="s">
-        <v>4317</v>
+        <v>4253</v>
       </c>
       <c r="C154" s="70" t="s">
         <v>31</v>
@@ -17598,7 +17583,7 @@
         <v>3484</v>
       </c>
       <c r="B155" s="70" t="s">
-        <v>4318</v>
+        <v>4254</v>
       </c>
       <c r="C155" s="70" t="s">
         <v>89</v>
@@ -17613,7 +17598,7 @@
         <v>3485</v>
       </c>
       <c r="B156" s="70" t="s">
-        <v>4319</v>
+        <v>4255</v>
       </c>
       <c r="C156" s="70" t="s">
         <v>31</v>
@@ -17630,7 +17615,7 @@
         <v>3486</v>
       </c>
       <c r="B157" s="70" t="s">
-        <v>4320</v>
+        <v>4256</v>
       </c>
       <c r="C157" s="70" t="s">
         <v>89</v>
@@ -17645,7 +17630,7 @@
         <v>3487</v>
       </c>
       <c r="B158" s="70" t="s">
-        <v>4417</v>
+        <v>4321</v>
       </c>
       <c r="C158" s="70" t="s">
         <v>31</v>
@@ -17662,7 +17647,7 @@
         <v>3488</v>
       </c>
       <c r="B159" s="70" t="s">
-        <v>4321</v>
+        <v>4257</v>
       </c>
       <c r="C159" s="70" t="s">
         <v>89</v>
@@ -17677,7 +17662,7 @@
         <v>3489</v>
       </c>
       <c r="B160" s="70" t="s">
-        <v>4322</v>
+        <v>4258</v>
       </c>
       <c r="C160" s="70" t="s">
         <v>31</v>
@@ -17694,7 +17679,7 @@
         <v>3490</v>
       </c>
       <c r="B161" s="70" t="s">
-        <v>4323</v>
+        <v>4259</v>
       </c>
       <c r="C161" s="70" t="s">
         <v>89</v>
@@ -17709,7 +17694,7 @@
         <v>3491</v>
       </c>
       <c r="B162" s="70" t="s">
-        <v>4324</v>
+        <v>4260</v>
       </c>
       <c r="C162" s="70" t="s">
         <v>31</v>
@@ -17726,7 +17711,7 @@
         <v>3492</v>
       </c>
       <c r="B163" s="70" t="s">
-        <v>4325</v>
+        <v>4261</v>
       </c>
       <c r="C163" s="70" t="s">
         <v>89</v>
@@ -17741,7 +17726,7 @@
         <v>3493</v>
       </c>
       <c r="B164" s="70" t="s">
-        <v>4326</v>
+        <v>4262</v>
       </c>
       <c r="C164" s="70" t="s">
         <v>31</v>
@@ -17758,7 +17743,7 @@
         <v>3494</v>
       </c>
       <c r="B165" s="70" t="s">
-        <v>4327</v>
+        <v>4263</v>
       </c>
       <c r="C165" s="70" t="s">
         <v>89</v>
@@ -17773,7 +17758,7 @@
         <v>3495</v>
       </c>
       <c r="B166" s="70" t="s">
-        <v>4328</v>
+        <v>4264</v>
       </c>
       <c r="C166" s="70" t="s">
         <v>31</v>
@@ -17790,7 +17775,7 @@
         <v>3496</v>
       </c>
       <c r="B167" s="70" t="s">
-        <v>4329</v>
+        <v>4265</v>
       </c>
       <c r="C167" s="70" t="s">
         <v>89</v>
@@ -17805,7 +17790,7 @@
         <v>3497</v>
       </c>
       <c r="B168" s="70" t="s">
-        <v>4330</v>
+        <v>4266</v>
       </c>
       <c r="C168" s="70" t="s">
         <v>31</v>
@@ -17822,7 +17807,7 @@
         <v>3498</v>
       </c>
       <c r="B169" s="72" t="s">
-        <v>4331</v>
+        <v>4267</v>
       </c>
       <c r="C169" s="72" t="s">
         <v>89</v>
@@ -17837,7 +17822,7 @@
         <v>3499</v>
       </c>
       <c r="B170" s="72" t="s">
-        <v>4332</v>
+        <v>4268</v>
       </c>
       <c r="C170" s="72" t="s">
         <v>31</v>
@@ -17854,7 +17839,7 @@
         <v>3500</v>
       </c>
       <c r="B171" s="72" t="s">
-        <v>4333</v>
+        <v>4269</v>
       </c>
       <c r="C171" s="72" t="s">
         <v>89</v>
@@ -17869,7 +17854,7 @@
         <v>3501</v>
       </c>
       <c r="B172" s="72" t="s">
-        <v>4334</v>
+        <v>4270</v>
       </c>
       <c r="C172" s="72" t="s">
         <v>31</v>
@@ -17886,7 +17871,7 @@
         <v>3502</v>
       </c>
       <c r="B173" s="72" t="s">
-        <v>4335</v>
+        <v>4271</v>
       </c>
       <c r="C173" s="72" t="s">
         <v>89</v>
@@ -17901,7 +17886,7 @@
         <v>3503</v>
       </c>
       <c r="B174" s="72" t="s">
-        <v>4336</v>
+        <v>4272</v>
       </c>
       <c r="C174" s="72" t="s">
         <v>31</v>
@@ -17918,7 +17903,7 @@
         <v>3504</v>
       </c>
       <c r="B175" s="74" t="s">
-        <v>4337</v>
+        <v>4273</v>
       </c>
       <c r="C175" s="74" t="s">
         <v>89</v>
@@ -17933,7 +17918,7 @@
         <v>3505</v>
       </c>
       <c r="B176" s="74" t="s">
-        <v>4338</v>
+        <v>4274</v>
       </c>
       <c r="C176" s="74" t="s">
         <v>31</v>
@@ -17950,7 +17935,7 @@
         <v>3506</v>
       </c>
       <c r="B177" s="76" t="s">
-        <v>4339</v>
+        <v>4275</v>
       </c>
       <c r="C177" s="142" t="s">
         <v>89</v>
@@ -17965,7 +17950,7 @@
         <v>3507</v>
       </c>
       <c r="B178" s="76" t="s">
-        <v>4340</v>
+        <v>4276</v>
       </c>
       <c r="C178" s="142" t="s">
         <v>31</v>
@@ -17982,7 +17967,7 @@
         <v>3508</v>
       </c>
       <c r="B179" s="76" t="s">
-        <v>4341</v>
+        <v>4277</v>
       </c>
       <c r="C179" s="142" t="s">
         <v>89</v>
@@ -17997,7 +17982,7 @@
         <v>3509</v>
       </c>
       <c r="B180" s="76" t="s">
-        <v>4342</v>
+        <v>4278</v>
       </c>
       <c r="C180" s="142" t="s">
         <v>31</v>
@@ -18014,7 +17999,7 @@
         <v>3510</v>
       </c>
       <c r="B181" s="76" t="s">
-        <v>4343</v>
+        <v>4279</v>
       </c>
       <c r="C181" s="142" t="s">
         <v>89</v>
@@ -18029,7 +18014,7 @@
         <v>3511</v>
       </c>
       <c r="B182" s="76" t="s">
-        <v>4344</v>
+        <v>4280</v>
       </c>
       <c r="C182" s="142" t="s">
         <v>31</v>
@@ -20745,7 +20730,7 @@
         <v>1645</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>4561</v>
+        <v>4401</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -20777,7 +20762,7 @@
         <v>1649</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>4560</v>
+        <v>4400</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -21451,7 +21436,7 @@
         <v>1737</v>
       </c>
       <c r="B167" s="100" t="s">
-        <v>4418</v>
+        <v>4322</v>
       </c>
       <c r="C167" s="132" t="s">
         <v>201</v>
@@ -22946,7 +22931,7 @@
         <v>3534</v>
       </c>
       <c r="B6" s="104" t="s">
-        <v>4346</v>
+        <v>4466</v>
       </c>
       <c r="C6" s="52" t="s">
         <v>31</v>
@@ -22961,7 +22946,7 @@
         <v>3535</v>
       </c>
       <c r="B7" s="104" t="s">
-        <v>4347</v>
+        <v>4467</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>31</v>
@@ -22976,7 +22961,7 @@
         <v>3536</v>
       </c>
       <c r="B8" s="104" t="s">
-        <v>4348</v>
+        <v>4468</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>89</v>
@@ -22991,7 +22976,7 @@
         <v>3537</v>
       </c>
       <c r="B9" s="104" t="s">
-        <v>4349</v>
+        <v>4469</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>31</v>
@@ -23040,7 +23025,7 @@
         <v>3540</v>
       </c>
       <c r="B12" s="104" t="s">
-        <v>4345</v>
+        <v>4470</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>37</v>
@@ -23055,7 +23040,7 @@
         <v>3541</v>
       </c>
       <c r="B13" s="104" t="s">
-        <v>4350</v>
+        <v>4471</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>37</v>
@@ -23070,7 +23055,7 @@
         <v>3542</v>
       </c>
       <c r="B14" s="104" t="s">
-        <v>4351</v>
+        <v>4472</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>37</v>
@@ -23085,7 +23070,7 @@
         <v>3543</v>
       </c>
       <c r="B15" s="104" t="s">
-        <v>4352</v>
+        <v>4473</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>47</v>
@@ -23100,7 +23085,7 @@
         <v>3544</v>
       </c>
       <c r="B16" s="104" t="s">
-        <v>4353</v>
+        <v>4474</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>47</v>
@@ -23115,7 +23100,7 @@
         <v>3545</v>
       </c>
       <c r="B17" s="104" t="s">
-        <v>4354</v>
+        <v>4475</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>37</v>
@@ -23130,7 +23115,7 @@
         <v>3546</v>
       </c>
       <c r="B18" s="104" t="s">
-        <v>4355</v>
+        <v>4498</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>47</v>
@@ -23145,7 +23130,7 @@
         <v>3547</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>4356</v>
+        <v>4476</v>
       </c>
       <c r="C19" s="122" t="s">
         <v>197</v>
@@ -23160,7 +23145,7 @@
         <v>3548</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>4357</v>
+        <v>4477</v>
       </c>
       <c r="C20" s="122" t="s">
         <v>201</v>
@@ -23177,7 +23162,7 @@
         <v>3549</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>4358</v>
+        <v>4478</v>
       </c>
       <c r="C21" s="122" t="s">
         <v>197</v>
@@ -23192,7 +23177,7 @@
         <v>3550</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>4359</v>
+        <v>4479</v>
       </c>
       <c r="C22" s="122" t="s">
         <v>201</v>
@@ -23209,7 +23194,7 @@
         <v>3551</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>4360</v>
+        <v>4480</v>
       </c>
       <c r="C23" s="122" t="s">
         <v>197</v>
@@ -23224,7 +23209,7 @@
         <v>3552</v>
       </c>
       <c r="B24" s="60" t="s">
-        <v>4361</v>
+        <v>4481</v>
       </c>
       <c r="C24" s="122" t="s">
         <v>201</v>
@@ -23241,7 +23226,7 @@
         <v>3553</v>
       </c>
       <c r="B25" s="60" t="s">
-        <v>4362</v>
+        <v>4482</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>197</v>
@@ -23256,7 +23241,7 @@
         <v>3554</v>
       </c>
       <c r="B26" s="60" t="s">
-        <v>4363</v>
+        <v>4483</v>
       </c>
       <c r="C26" s="122" t="s">
         <v>201</v>
@@ -23273,7 +23258,7 @@
         <v>3555</v>
       </c>
       <c r="B27" s="60" t="s">
-        <v>4364</v>
+        <v>4484</v>
       </c>
       <c r="C27" s="122" t="s">
         <v>197</v>
@@ -23288,7 +23273,7 @@
         <v>3556</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>4365</v>
+        <v>4485</v>
       </c>
       <c r="C28" s="122" t="s">
         <v>201</v>
@@ -23305,7 +23290,7 @@
         <v>3557</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>4366</v>
+        <v>4486</v>
       </c>
       <c r="C29" s="122" t="s">
         <v>197</v>
@@ -23320,7 +23305,7 @@
         <v>3558</v>
       </c>
       <c r="B30" s="60" t="s">
-        <v>4367</v>
+        <v>4487</v>
       </c>
       <c r="C30" s="122" t="s">
         <v>201</v>
@@ -23337,7 +23322,7 @@
         <v>3559</v>
       </c>
       <c r="B31" s="60" t="s">
-        <v>4368</v>
+        <v>4488</v>
       </c>
       <c r="C31" s="122" t="s">
         <v>197</v>
@@ -23352,7 +23337,7 @@
         <v>3560</v>
       </c>
       <c r="B32" s="60" t="s">
-        <v>4369</v>
+        <v>1646</v>
       </c>
       <c r="C32" s="122" t="s">
         <v>201</v>
@@ -23369,7 +23354,7 @@
         <v>3561</v>
       </c>
       <c r="B33" s="62" t="s">
-        <v>4370</v>
+        <v>4489</v>
       </c>
       <c r="C33" s="123" t="s">
         <v>201</v>
@@ -23384,7 +23369,7 @@
         <v>3562</v>
       </c>
       <c r="B34" s="62" t="s">
-        <v>4371</v>
+        <v>4490</v>
       </c>
       <c r="C34" s="123" t="s">
         <v>201</v>
@@ -23399,7 +23384,7 @@
         <v>3563</v>
       </c>
       <c r="B35" s="62" t="s">
-        <v>4372</v>
+        <v>4491</v>
       </c>
       <c r="C35" s="123" t="s">
         <v>201</v>
@@ -23414,7 +23399,7 @@
         <v>3564</v>
       </c>
       <c r="B36" s="62" t="s">
-        <v>4373</v>
+        <v>4492</v>
       </c>
       <c r="C36" s="123" t="s">
         <v>201</v>
@@ -23429,7 +23414,7 @@
         <v>3565</v>
       </c>
       <c r="B37" s="62" t="s">
-        <v>4374</v>
+        <v>4493</v>
       </c>
       <c r="C37" s="123" t="s">
         <v>201</v>
@@ -23444,7 +23429,7 @@
         <v>3566</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>4375</v>
+        <v>4494</v>
       </c>
       <c r="C38" s="123" t="s">
         <v>201</v>
@@ -23459,7 +23444,7 @@
         <v>3567</v>
       </c>
       <c r="B39" s="62" t="s">
-        <v>4376</v>
+        <v>4495</v>
       </c>
       <c r="C39" s="123" t="s">
         <v>201</v>
@@ -24481,7 +24466,7 @@
         <v>3631</v>
       </c>
       <c r="B103" s="96" t="s">
-        <v>1646</v>
+        <v>4401</v>
       </c>
       <c r="C103" s="130" t="s">
         <v>201</v>
@@ -25095,7 +25080,7 @@
         <v>3671</v>
       </c>
       <c r="B143" s="100" t="s">
-        <v>4418</v>
+        <v>4322</v>
       </c>
       <c r="C143" s="132" t="s">
         <v>201</v>
@@ -25144,7 +25129,7 @@
         <v>3674</v>
       </c>
       <c r="B146" s="106" t="s">
-        <v>4377</v>
+        <v>4281</v>
       </c>
       <c r="C146" s="70" t="s">
         <v>89</v>
@@ -25159,7 +25144,7 @@
         <v>3675</v>
       </c>
       <c r="B147" s="106" t="s">
-        <v>4378</v>
+        <v>4282</v>
       </c>
       <c r="C147" s="70" t="s">
         <v>31</v>
@@ -25176,7 +25161,7 @@
         <v>3676</v>
       </c>
       <c r="B148" s="106" t="s">
-        <v>4379</v>
+        <v>4283</v>
       </c>
       <c r="C148" s="70" t="s">
         <v>89</v>
@@ -25191,7 +25176,7 @@
         <v>3677</v>
       </c>
       <c r="B149" s="106" t="s">
-        <v>4380</v>
+        <v>4284</v>
       </c>
       <c r="C149" s="70" t="s">
         <v>31</v>
@@ -25208,7 +25193,7 @@
         <v>3678</v>
       </c>
       <c r="B150" s="106" t="s">
-        <v>4381</v>
+        <v>4285</v>
       </c>
       <c r="C150" s="70" t="s">
         <v>89</v>
@@ -25223,7 +25208,7 @@
         <v>3679</v>
       </c>
       <c r="B151" s="106" t="s">
-        <v>4382</v>
+        <v>4286</v>
       </c>
       <c r="C151" s="70" t="s">
         <v>31</v>
@@ -25240,7 +25225,7 @@
         <v>3680</v>
       </c>
       <c r="B152" s="106" t="s">
-        <v>4383</v>
+        <v>4287</v>
       </c>
       <c r="C152" s="70" t="s">
         <v>89</v>
@@ -25255,7 +25240,7 @@
         <v>3681</v>
       </c>
       <c r="B153" s="106" t="s">
-        <v>4384</v>
+        <v>4288</v>
       </c>
       <c r="C153" s="70" t="s">
         <v>31</v>
@@ -25272,7 +25257,7 @@
         <v>3682</v>
       </c>
       <c r="B154" s="106" t="s">
-        <v>4385</v>
+        <v>4289</v>
       </c>
       <c r="C154" s="70" t="s">
         <v>89</v>
@@ -25287,7 +25272,7 @@
         <v>3683</v>
       </c>
       <c r="B155" s="106" t="s">
-        <v>4386</v>
+        <v>4290</v>
       </c>
       <c r="C155" s="70" t="s">
         <v>31</v>
@@ -25304,7 +25289,7 @@
         <v>3684</v>
       </c>
       <c r="B156" s="106" t="s">
-        <v>4387</v>
+        <v>4291</v>
       </c>
       <c r="C156" s="70" t="s">
         <v>89</v>
@@ -25319,7 +25304,7 @@
         <v>3685</v>
       </c>
       <c r="B157" s="106" t="s">
-        <v>4388</v>
+        <v>4292</v>
       </c>
       <c r="C157" s="70" t="s">
         <v>31</v>
@@ -25336,7 +25321,7 @@
         <v>3686</v>
       </c>
       <c r="B158" s="106" t="s">
-        <v>4389</v>
+        <v>4293</v>
       </c>
       <c r="C158" s="70" t="s">
         <v>89</v>
@@ -25351,7 +25336,7 @@
         <v>3687</v>
       </c>
       <c r="B159" s="106" t="s">
-        <v>4390</v>
+        <v>4294</v>
       </c>
       <c r="C159" s="70" t="s">
         <v>31</v>
@@ -25368,7 +25353,7 @@
         <v>3688</v>
       </c>
       <c r="B160" s="106" t="s">
-        <v>4391</v>
+        <v>4295</v>
       </c>
       <c r="C160" s="70" t="s">
         <v>89</v>
@@ -25383,7 +25368,7 @@
         <v>3689</v>
       </c>
       <c r="B161" s="106" t="s">
-        <v>4392</v>
+        <v>4296</v>
       </c>
       <c r="C161" s="70" t="s">
         <v>31</v>
@@ -25400,7 +25385,7 @@
         <v>3690</v>
       </c>
       <c r="B162" s="106" t="s">
-        <v>4393</v>
+        <v>4297</v>
       </c>
       <c r="C162" s="70" t="s">
         <v>89</v>
@@ -25415,7 +25400,7 @@
         <v>3691</v>
       </c>
       <c r="B163" s="106" t="s">
-        <v>4394</v>
+        <v>4298</v>
       </c>
       <c r="C163" s="70" t="s">
         <v>31</v>
@@ -25432,7 +25417,7 @@
         <v>3692</v>
       </c>
       <c r="B164" s="106" t="s">
-        <v>4395</v>
+        <v>4299</v>
       </c>
       <c r="C164" s="70" t="s">
         <v>89</v>
@@ -25447,7 +25432,7 @@
         <v>3693</v>
       </c>
       <c r="B165" s="106" t="s">
-        <v>4396</v>
+        <v>4300</v>
       </c>
       <c r="C165" s="70" t="s">
         <v>31</v>
@@ -25464,7 +25449,7 @@
         <v>3694</v>
       </c>
       <c r="B166" s="106" t="s">
-        <v>4397</v>
+        <v>4301</v>
       </c>
       <c r="C166" s="70" t="s">
         <v>89</v>
@@ -25479,7 +25464,7 @@
         <v>3695</v>
       </c>
       <c r="B167" s="106" t="s">
-        <v>4398</v>
+        <v>4302</v>
       </c>
       <c r="C167" s="70" t="s">
         <v>31</v>
@@ -25496,7 +25481,7 @@
         <v>3696</v>
       </c>
       <c r="B168" s="108" t="s">
-        <v>4399</v>
+        <v>4303</v>
       </c>
       <c r="C168" s="72" t="s">
         <v>89</v>
@@ -25511,7 +25496,7 @@
         <v>3697</v>
       </c>
       <c r="B169" s="108" t="s">
-        <v>4400</v>
+        <v>4304</v>
       </c>
       <c r="C169" s="72" t="s">
         <v>31</v>
@@ -25528,7 +25513,7 @@
         <v>3698</v>
       </c>
       <c r="B170" s="108" t="s">
-        <v>4401</v>
+        <v>4305</v>
       </c>
       <c r="C170" s="72" t="s">
         <v>89</v>
@@ -25543,7 +25528,7 @@
         <v>3699</v>
       </c>
       <c r="B171" s="108" t="s">
-        <v>4402</v>
+        <v>4306</v>
       </c>
       <c r="C171" s="72" t="s">
         <v>31</v>
@@ -25560,7 +25545,7 @@
         <v>3700</v>
       </c>
       <c r="B172" s="108" t="s">
-        <v>4403</v>
+        <v>4307</v>
       </c>
       <c r="C172" s="72" t="s">
         <v>89</v>
@@ -25575,7 +25560,7 @@
         <v>3701</v>
       </c>
       <c r="B173" s="108" t="s">
-        <v>4404</v>
+        <v>4308</v>
       </c>
       <c r="C173" s="72" t="s">
         <v>31</v>
@@ -25592,7 +25577,7 @@
         <v>3702</v>
       </c>
       <c r="B174" s="110" t="s">
-        <v>4405</v>
+        <v>4309</v>
       </c>
       <c r="C174" s="74" t="s">
         <v>89</v>
@@ -25607,7 +25592,7 @@
         <v>3703</v>
       </c>
       <c r="B175" s="110" t="s">
-        <v>4406</v>
+        <v>4310</v>
       </c>
       <c r="C175" s="74" t="s">
         <v>31</v>
@@ -25624,7 +25609,7 @@
         <v>3704</v>
       </c>
       <c r="B176" s="112" t="s">
-        <v>4407</v>
+        <v>4311</v>
       </c>
       <c r="C176" s="142" t="s">
         <v>89</v>
@@ -25639,7 +25624,7 @@
         <v>3705</v>
       </c>
       <c r="B177" s="112" t="s">
-        <v>4408</v>
+        <v>4312</v>
       </c>
       <c r="C177" s="142" t="s">
         <v>31</v>
@@ -25656,7 +25641,7 @@
         <v>3706</v>
       </c>
       <c r="B178" s="112" t="s">
-        <v>4409</v>
+        <v>4313</v>
       </c>
       <c r="C178" s="142" t="s">
         <v>89</v>
@@ -25671,7 +25656,7 @@
         <v>3707</v>
       </c>
       <c r="B179" s="112" t="s">
-        <v>4410</v>
+        <v>4314</v>
       </c>
       <c r="C179" s="142" t="s">
         <v>31</v>
@@ -25688,7 +25673,7 @@
         <v>3708</v>
       </c>
       <c r="B180" s="112" t="s">
-        <v>4411</v>
+        <v>4315</v>
       </c>
       <c r="C180" s="142" t="s">
         <v>89</v>
@@ -25703,7 +25688,7 @@
         <v>3709</v>
       </c>
       <c r="B181" s="112" t="s">
-        <v>4412</v>
+        <v>4316</v>
       </c>
       <c r="C181" s="142" t="s">
         <v>31</v>
@@ -28420,7 +28405,7 @@
         <v>2134</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>4562</v>
+        <v>4402</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -28452,7 +28437,7 @@
         <v>2138</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>4563</v>
+        <v>4403</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -30632,7 +30617,7 @@
         <v>3734</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>4419</v>
+        <v>4499</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>31</v>
@@ -30647,7 +30632,7 @@
         <v>3735</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>4420</v>
+        <v>4500</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>31</v>
@@ -30662,7 +30647,7 @@
         <v>3736</v>
       </c>
       <c r="B9" s="52" t="s">
-        <v>4421</v>
+        <v>4501</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>89</v>
@@ -30677,7 +30662,7 @@
         <v>3737</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>4422</v>
+        <v>4502</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>31</v>
@@ -30726,7 +30711,7 @@
         <v>3740</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>4423</v>
+        <v>4503</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>37</v>
@@ -30741,7 +30726,7 @@
         <v>3741</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>4424</v>
+        <v>4504</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>37</v>
@@ -30756,7 +30741,7 @@
         <v>3742</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>4425</v>
+        <v>4505</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>37</v>
@@ -30771,7 +30756,7 @@
         <v>3743</v>
       </c>
       <c r="B16" s="52" t="s">
-        <v>4426</v>
+        <v>4506</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>47</v>
@@ -30786,7 +30771,7 @@
         <v>3744</v>
       </c>
       <c r="B17" s="52" t="s">
-        <v>4427</v>
+        <v>4507</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>47</v>
@@ -30801,7 +30786,7 @@
         <v>3745</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>4428</v>
+        <v>4508</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>37</v>
@@ -30816,7 +30801,7 @@
         <v>3746</v>
       </c>
       <c r="B19" s="52" t="s">
-        <v>4429</v>
+        <v>4509</v>
       </c>
       <c r="C19" s="52" t="s">
         <v>47</v>
@@ -30831,7 +30816,7 @@
         <v>3747</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>4430</v>
+        <v>4510</v>
       </c>
       <c r="C20" s="122" t="s">
         <v>197</v>
@@ -30846,7 +30831,7 @@
         <v>3748</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>4431</v>
+        <v>4511</v>
       </c>
       <c r="C21" s="122" t="s">
         <v>201</v>
@@ -30863,7 +30848,7 @@
         <v>3749</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>4432</v>
+        <v>4512</v>
       </c>
       <c r="C22" s="122" t="s">
         <v>197</v>
@@ -30878,7 +30863,7 @@
         <v>3750</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>4433</v>
+        <v>4513</v>
       </c>
       <c r="C23" s="122" t="s">
         <v>201</v>
@@ -30895,7 +30880,7 @@
         <v>3751</v>
       </c>
       <c r="B24" s="60" t="s">
-        <v>4434</v>
+        <v>4514</v>
       </c>
       <c r="C24" s="122" t="s">
         <v>197</v>
@@ -30910,7 +30895,7 @@
         <v>3752</v>
       </c>
       <c r="B25" s="60" t="s">
-        <v>4435</v>
+        <v>4515</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>201</v>
@@ -30927,7 +30912,7 @@
         <v>3753</v>
       </c>
       <c r="B26" s="60" t="s">
-        <v>4436</v>
+        <v>4516</v>
       </c>
       <c r="C26" s="122" t="s">
         <v>197</v>
@@ -30942,7 +30927,7 @@
         <v>3754</v>
       </c>
       <c r="B27" s="60" t="s">
-        <v>4437</v>
+        <v>4517</v>
       </c>
       <c r="C27" s="122" t="s">
         <v>201</v>
@@ -30959,7 +30944,7 @@
         <v>3755</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>4438</v>
+        <v>4518</v>
       </c>
       <c r="C28" s="122" t="s">
         <v>197</v>
@@ -30974,7 +30959,7 @@
         <v>3756</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>4439</v>
+        <v>4519</v>
       </c>
       <c r="C29" s="122" t="s">
         <v>201</v>
@@ -30991,7 +30976,7 @@
         <v>3757</v>
       </c>
       <c r="B30" s="60" t="s">
-        <v>4440</v>
+        <v>4520</v>
       </c>
       <c r="C30" s="122" t="s">
         <v>197</v>
@@ -31006,7 +30991,7 @@
         <v>3758</v>
       </c>
       <c r="B31" s="60" t="s">
-        <v>4441</v>
+        <v>4521</v>
       </c>
       <c r="C31" s="122" t="s">
         <v>201</v>
@@ -31023,7 +31008,7 @@
         <v>3759</v>
       </c>
       <c r="B32" s="60" t="s">
-        <v>4442</v>
+        <v>4522</v>
       </c>
       <c r="C32" s="122" t="s">
         <v>197</v>
@@ -31038,7 +31023,7 @@
         <v>3760</v>
       </c>
       <c r="B33" s="60" t="s">
-        <v>4443</v>
+        <v>2135</v>
       </c>
       <c r="C33" s="122" t="s">
         <v>201</v>
@@ -31055,7 +31040,7 @@
         <v>3761</v>
       </c>
       <c r="B34" s="62" t="s">
-        <v>4444</v>
+        <v>4523</v>
       </c>
       <c r="C34" s="123" t="s">
         <v>201</v>
@@ -31070,7 +31055,7 @@
         <v>3762</v>
       </c>
       <c r="B35" s="62" t="s">
-        <v>4445</v>
+        <v>4524</v>
       </c>
       <c r="C35" s="123" t="s">
         <v>201</v>
@@ -31085,7 +31070,7 @@
         <v>3763</v>
       </c>
       <c r="B36" s="62" t="s">
-        <v>4446</v>
+        <v>4525</v>
       </c>
       <c r="C36" s="123" t="s">
         <v>201</v>
@@ -31100,7 +31085,7 @@
         <v>3764</v>
       </c>
       <c r="B37" s="62" t="s">
-        <v>4447</v>
+        <v>4526</v>
       </c>
       <c r="C37" s="123" t="s">
         <v>201</v>
@@ -31115,7 +31100,7 @@
         <v>3765</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>4448</v>
+        <v>4527</v>
       </c>
       <c r="C38" s="123" t="s">
         <v>201</v>
@@ -31130,7 +31115,7 @@
         <v>3766</v>
       </c>
       <c r="B39" s="62" t="s">
-        <v>4449</v>
+        <v>4528</v>
       </c>
       <c r="C39" s="123" t="s">
         <v>201</v>
@@ -31145,7 +31130,7 @@
         <v>3767</v>
       </c>
       <c r="B40" s="62" t="s">
-        <v>4450</v>
+        <v>4529</v>
       </c>
       <c r="C40" s="123" t="s">
         <v>201</v>
@@ -32167,7 +32152,7 @@
         <v>3831</v>
       </c>
       <c r="B104" s="96" t="s">
-        <v>2135</v>
+        <v>4402</v>
       </c>
       <c r="C104" s="130" t="s">
         <v>201</v>
@@ -32830,7 +32815,7 @@
         <v>3874</v>
       </c>
       <c r="B147" s="70" t="s">
-        <v>4451</v>
+        <v>4323</v>
       </c>
       <c r="C147" s="70" t="s">
         <v>89</v>
@@ -32845,7 +32830,7 @@
         <v>3875</v>
       </c>
       <c r="B148" s="70" t="s">
-        <v>4452</v>
+        <v>4324</v>
       </c>
       <c r="C148" s="70" t="s">
         <v>31</v>
@@ -32862,7 +32847,7 @@
         <v>3876</v>
       </c>
       <c r="B149" s="70" t="s">
-        <v>4453</v>
+        <v>4325</v>
       </c>
       <c r="C149" s="70" t="s">
         <v>89</v>
@@ -32877,7 +32862,7 @@
         <v>3877</v>
       </c>
       <c r="B150" s="70" t="s">
-        <v>4454</v>
+        <v>4326</v>
       </c>
       <c r="C150" s="70" t="s">
         <v>31</v>
@@ -32894,7 +32879,7 @@
         <v>3878</v>
       </c>
       <c r="B151" s="70" t="s">
-        <v>4455</v>
+        <v>4327</v>
       </c>
       <c r="C151" s="70" t="s">
         <v>89</v>
@@ -32909,7 +32894,7 @@
         <v>3879</v>
       </c>
       <c r="B152" s="70" t="s">
-        <v>4456</v>
+        <v>4328</v>
       </c>
       <c r="C152" s="70" t="s">
         <v>31</v>
@@ -32926,7 +32911,7 @@
         <v>3880</v>
       </c>
       <c r="B153" s="70" t="s">
-        <v>4457</v>
+        <v>4329</v>
       </c>
       <c r="C153" s="70" t="s">
         <v>89</v>
@@ -32941,7 +32926,7 @@
         <v>3881</v>
       </c>
       <c r="B154" s="70" t="s">
-        <v>4458</v>
+        <v>4330</v>
       </c>
       <c r="C154" s="70" t="s">
         <v>31</v>
@@ -32958,7 +32943,7 @@
         <v>3882</v>
       </c>
       <c r="B155" s="70" t="s">
-        <v>4459</v>
+        <v>4331</v>
       </c>
       <c r="C155" s="70" t="s">
         <v>89</v>
@@ -32973,7 +32958,7 @@
         <v>3883</v>
       </c>
       <c r="B156" s="70" t="s">
-        <v>4460</v>
+        <v>4332</v>
       </c>
       <c r="C156" s="70" t="s">
         <v>31</v>
@@ -32990,7 +32975,7 @@
         <v>3884</v>
       </c>
       <c r="B157" s="70" t="s">
-        <v>4461</v>
+        <v>4333</v>
       </c>
       <c r="C157" s="70" t="s">
         <v>89</v>
@@ -33005,7 +32990,7 @@
         <v>3885</v>
       </c>
       <c r="B158" s="70" t="s">
-        <v>4462</v>
+        <v>4334</v>
       </c>
       <c r="C158" s="70" t="s">
         <v>31</v>
@@ -33022,7 +33007,7 @@
         <v>3886</v>
       </c>
       <c r="B159" s="70" t="s">
-        <v>4463</v>
+        <v>4335</v>
       </c>
       <c r="C159" s="70" t="s">
         <v>89</v>
@@ -33037,7 +33022,7 @@
         <v>3887</v>
       </c>
       <c r="B160" s="70" t="s">
-        <v>4464</v>
+        <v>4336</v>
       </c>
       <c r="C160" s="70" t="s">
         <v>31</v>
@@ -33054,7 +33039,7 @@
         <v>3888</v>
       </c>
       <c r="B161" s="70" t="s">
-        <v>4465</v>
+        <v>4337</v>
       </c>
       <c r="C161" s="70" t="s">
         <v>89</v>
@@ -33069,7 +33054,7 @@
         <v>3889</v>
       </c>
       <c r="B162" s="70" t="s">
-        <v>4466</v>
+        <v>4338</v>
       </c>
       <c r="C162" s="70" t="s">
         <v>31</v>
@@ -33086,7 +33071,7 @@
         <v>3890</v>
       </c>
       <c r="B163" s="70" t="s">
-        <v>4467</v>
+        <v>4339</v>
       </c>
       <c r="C163" s="70" t="s">
         <v>89</v>
@@ -33101,7 +33086,7 @@
         <v>3891</v>
       </c>
       <c r="B164" s="70" t="s">
-        <v>4468</v>
+        <v>4340</v>
       </c>
       <c r="C164" s="70" t="s">
         <v>31</v>
@@ -33118,7 +33103,7 @@
         <v>3892</v>
       </c>
       <c r="B165" s="70" t="s">
-        <v>4469</v>
+        <v>4341</v>
       </c>
       <c r="C165" s="70" t="s">
         <v>89</v>
@@ -33133,7 +33118,7 @@
         <v>3893</v>
       </c>
       <c r="B166" s="70" t="s">
-        <v>4470</v>
+        <v>4342</v>
       </c>
       <c r="C166" s="70" t="s">
         <v>31</v>
@@ -33150,7 +33135,7 @@
         <v>3894</v>
       </c>
       <c r="B167" s="70" t="s">
-        <v>4471</v>
+        <v>4343</v>
       </c>
       <c r="C167" s="70" t="s">
         <v>89</v>
@@ -33165,7 +33150,7 @@
         <v>3895</v>
       </c>
       <c r="B168" s="70" t="s">
-        <v>4472</v>
+        <v>4344</v>
       </c>
       <c r="C168" s="70" t="s">
         <v>31</v>
@@ -33182,7 +33167,7 @@
         <v>3896</v>
       </c>
       <c r="B169" s="72" t="s">
-        <v>4473</v>
+        <v>4345</v>
       </c>
       <c r="C169" s="72" t="s">
         <v>89</v>
@@ -33197,7 +33182,7 @@
         <v>3897</v>
       </c>
       <c r="B170" s="72" t="s">
-        <v>4474</v>
+        <v>4346</v>
       </c>
       <c r="C170" s="72" t="s">
         <v>31</v>
@@ -33214,7 +33199,7 @@
         <v>3898</v>
       </c>
       <c r="B171" s="72" t="s">
-        <v>4475</v>
+        <v>4347</v>
       </c>
       <c r="C171" s="72" t="s">
         <v>89</v>
@@ -33229,7 +33214,7 @@
         <v>3899</v>
       </c>
       <c r="B172" s="72" t="s">
-        <v>4476</v>
+        <v>4348</v>
       </c>
       <c r="C172" s="72" t="s">
         <v>31</v>
@@ -33246,7 +33231,7 @@
         <v>3900</v>
       </c>
       <c r="B173" s="72" t="s">
-        <v>4477</v>
+        <v>4349</v>
       </c>
       <c r="C173" s="72" t="s">
         <v>89</v>
@@ -33261,7 +33246,7 @@
         <v>3901</v>
       </c>
       <c r="B174" s="72" t="s">
-        <v>4478</v>
+        <v>4350</v>
       </c>
       <c r="C174" s="72" t="s">
         <v>31</v>
@@ -33278,7 +33263,7 @@
         <v>3902</v>
       </c>
       <c r="B175" s="74" t="s">
-        <v>4479</v>
+        <v>4351</v>
       </c>
       <c r="C175" s="74" t="s">
         <v>89</v>
@@ -33293,7 +33278,7 @@
         <v>3903</v>
       </c>
       <c r="B176" s="74" t="s">
-        <v>4480</v>
+        <v>4352</v>
       </c>
       <c r="C176" s="74" t="s">
         <v>31</v>
@@ -33310,7 +33295,7 @@
         <v>3904</v>
       </c>
       <c r="B177" s="76" t="s">
-        <v>4481</v>
+        <v>4353</v>
       </c>
       <c r="C177" s="142" t="s">
         <v>89</v>
@@ -33325,7 +33310,7 @@
         <v>3905</v>
       </c>
       <c r="B178" s="76" t="s">
-        <v>4482</v>
+        <v>4354</v>
       </c>
       <c r="C178" s="142" t="s">
         <v>31</v>
@@ -33342,7 +33327,7 @@
         <v>3906</v>
       </c>
       <c r="B179" s="76" t="s">
-        <v>4483</v>
+        <v>4355</v>
       </c>
       <c r="C179" s="142" t="s">
         <v>89</v>
@@ -33357,7 +33342,7 @@
         <v>3907</v>
       </c>
       <c r="B180" s="76" t="s">
-        <v>4484</v>
+        <v>4356</v>
       </c>
       <c r="C180" s="142" t="s">
         <v>31</v>
@@ -33374,7 +33359,7 @@
         <v>3908</v>
       </c>
       <c r="B181" s="76" t="s">
-        <v>4485</v>
+        <v>4357</v>
       </c>
       <c r="C181" s="142" t="s">
         <v>89</v>
@@ -33389,7 +33374,7 @@
         <v>3909</v>
       </c>
       <c r="B182" s="76" t="s">
-        <v>4486</v>
+        <v>4358</v>
       </c>
       <c r="C182" s="142" t="s">
         <v>31</v>
@@ -36084,7 +36069,7 @@
         <v>2622</v>
       </c>
       <c r="B119" s="96" t="s">
-        <v>4564</v>
+        <v>4404</v>
       </c>
       <c r="C119" s="130" t="s">
         <v>201</v>
@@ -36116,7 +36101,7 @@
         <v>2626</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>4565</v>
+        <v>4405</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -38274,7 +38259,7 @@
         <v>3932</v>
       </c>
       <c r="B5" s="52" t="s">
-        <v>4487</v>
+        <v>4530</v>
       </c>
       <c r="C5" s="52" t="s">
         <v>31</v>
@@ -38289,7 +38274,7 @@
         <v>3933</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>4488</v>
+        <v>4531</v>
       </c>
       <c r="C6" s="52" t="s">
         <v>31</v>
@@ -38304,7 +38289,7 @@
         <v>3934</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>4489</v>
+        <v>4532</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>89</v>
@@ -38319,7 +38304,7 @@
         <v>3935</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>4490</v>
+        <v>4533</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>31</v>
@@ -38368,7 +38353,7 @@
         <v>3938</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>4491</v>
+        <v>4534</v>
       </c>
       <c r="C11" s="52" t="s">
         <v>37</v>
@@ -38383,7 +38368,7 @@
         <v>3939</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>4492</v>
+        <v>4535</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>37</v>
@@ -38398,7 +38383,7 @@
         <v>3940</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>4493</v>
+        <v>4536</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>37</v>
@@ -38413,7 +38398,7 @@
         <v>3941</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>4494</v>
+        <v>4537</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>47</v>
@@ -38428,7 +38413,7 @@
         <v>3942</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>4495</v>
+        <v>4538</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>47</v>
@@ -38443,7 +38428,7 @@
         <v>3943</v>
       </c>
       <c r="B16" s="52" t="s">
-        <v>4496</v>
+        <v>4539</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>37</v>
@@ -38458,7 +38443,7 @@
         <v>3944</v>
       </c>
       <c r="B17" s="52" t="s">
-        <v>4497</v>
+        <v>4540</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>47</v>
@@ -38473,7 +38458,7 @@
         <v>3945</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>4498</v>
+        <v>4541</v>
       </c>
       <c r="C18" s="122" t="s">
         <v>197</v>
@@ -38488,7 +38473,7 @@
         <v>3946</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>4499</v>
+        <v>4542</v>
       </c>
       <c r="C19" s="122" t="s">
         <v>201</v>
@@ -38505,7 +38490,7 @@
         <v>3947</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>4500</v>
+        <v>4543</v>
       </c>
       <c r="C20" s="122" t="s">
         <v>197</v>
@@ -38520,7 +38505,7 @@
         <v>3948</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>4501</v>
+        <v>4544</v>
       </c>
       <c r="C21" s="122" t="s">
         <v>201</v>
@@ -38537,7 +38522,7 @@
         <v>3949</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>4502</v>
+        <v>4545</v>
       </c>
       <c r="C22" s="122" t="s">
         <v>197</v>
@@ -38552,7 +38537,7 @@
         <v>3950</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>4503</v>
+        <v>4546</v>
       </c>
       <c r="C23" s="122" t="s">
         <v>201</v>
@@ -38569,7 +38554,7 @@
         <v>3951</v>
       </c>
       <c r="B24" s="60" t="s">
-        <v>4504</v>
+        <v>4547</v>
       </c>
       <c r="C24" s="122" t="s">
         <v>197</v>
@@ -38584,7 +38569,7 @@
         <v>3952</v>
       </c>
       <c r="B25" s="60" t="s">
-        <v>4505</v>
+        <v>4548</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>201</v>
@@ -38601,7 +38586,7 @@
         <v>3953</v>
       </c>
       <c r="B26" s="60" t="s">
-        <v>4506</v>
+        <v>4549</v>
       </c>
       <c r="C26" s="122" t="s">
         <v>197</v>
@@ -38616,7 +38601,7 @@
         <v>3954</v>
       </c>
       <c r="B27" s="60" t="s">
-        <v>4507</v>
+        <v>4550</v>
       </c>
       <c r="C27" s="122" t="s">
         <v>201</v>
@@ -38633,7 +38618,7 @@
         <v>3955</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>4508</v>
+        <v>4551</v>
       </c>
       <c r="C28" s="122" t="s">
         <v>197</v>
@@ -38648,7 +38633,7 @@
         <v>3956</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>4509</v>
+        <v>4552</v>
       </c>
       <c r="C29" s="122" t="s">
         <v>201</v>
@@ -38665,7 +38650,7 @@
         <v>3957</v>
       </c>
       <c r="B30" s="60" t="s">
-        <v>4510</v>
+        <v>4553</v>
       </c>
       <c r="C30" s="122" t="s">
         <v>197</v>
@@ -38680,7 +38665,7 @@
         <v>3958</v>
       </c>
       <c r="B31" s="60" t="s">
-        <v>4511</v>
+        <v>2623</v>
       </c>
       <c r="C31" s="122" t="s">
         <v>201</v>
@@ -38697,7 +38682,7 @@
         <v>3959</v>
       </c>
       <c r="B32" s="62" t="s">
-        <v>4512</v>
+        <v>4554</v>
       </c>
       <c r="C32" s="123" t="s">
         <v>201</v>
@@ -38712,7 +38697,7 @@
         <v>3960</v>
       </c>
       <c r="B33" s="62" t="s">
-        <v>4513</v>
+        <v>4555</v>
       </c>
       <c r="C33" s="123" t="s">
         <v>201</v>
@@ -38727,7 +38712,7 @@
         <v>3961</v>
       </c>
       <c r="B34" s="62" t="s">
-        <v>4514</v>
+        <v>4556</v>
       </c>
       <c r="C34" s="123" t="s">
         <v>201</v>
@@ -38742,7 +38727,7 @@
         <v>3962</v>
       </c>
       <c r="B35" s="62" t="s">
-        <v>4515</v>
+        <v>4557</v>
       </c>
       <c r="C35" s="123" t="s">
         <v>201</v>
@@ -38757,7 +38742,7 @@
         <v>3963</v>
       </c>
       <c r="B36" s="62" t="s">
-        <v>4516</v>
+        <v>4558</v>
       </c>
       <c r="C36" s="123" t="s">
         <v>201</v>
@@ -38772,7 +38757,7 @@
         <v>3964</v>
       </c>
       <c r="B37" s="62" t="s">
-        <v>4517</v>
+        <v>4559</v>
       </c>
       <c r="C37" s="123" t="s">
         <v>201</v>
@@ -38787,7 +38772,7 @@
         <v>3965</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>4518</v>
+        <v>4560</v>
       </c>
       <c r="C38" s="123" t="s">
         <v>201</v>
@@ -39809,7 +39794,7 @@
         <v>4029</v>
       </c>
       <c r="B102" s="96" t="s">
-        <v>2623</v>
+        <v>4404</v>
       </c>
       <c r="C102" s="130" t="s">
         <v>201</v>
@@ -40472,7 +40457,7 @@
         <v>4072</v>
       </c>
       <c r="B145" s="70" t="s">
-        <v>4519</v>
+        <v>4359</v>
       </c>
       <c r="C145" s="70" t="s">
         <v>89</v>
@@ -40487,7 +40472,7 @@
         <v>4073</v>
       </c>
       <c r="B146" s="70" t="s">
-        <v>4520</v>
+        <v>4360</v>
       </c>
       <c r="C146" s="70" t="s">
         <v>31</v>
@@ -40504,7 +40489,7 @@
         <v>4074</v>
       </c>
       <c r="B147" s="70" t="s">
-        <v>4521</v>
+        <v>4361</v>
       </c>
       <c r="C147" s="70" t="s">
         <v>89</v>
@@ -40519,7 +40504,7 @@
         <v>4075</v>
       </c>
       <c r="B148" s="70" t="s">
-        <v>4522</v>
+        <v>4362</v>
       </c>
       <c r="C148" s="70" t="s">
         <v>31</v>
@@ -40536,7 +40521,7 @@
         <v>4076</v>
       </c>
       <c r="B149" s="70" t="s">
-        <v>4523</v>
+        <v>4363</v>
       </c>
       <c r="C149" s="70" t="s">
         <v>89</v>
@@ -40551,7 +40536,7 @@
         <v>4077</v>
       </c>
       <c r="B150" s="70" t="s">
-        <v>4524</v>
+        <v>4364</v>
       </c>
       <c r="C150" s="70" t="s">
         <v>31</v>
@@ -40568,7 +40553,7 @@
         <v>4078</v>
       </c>
       <c r="B151" s="70" t="s">
-        <v>4525</v>
+        <v>4365</v>
       </c>
       <c r="C151" s="70" t="s">
         <v>89</v>
@@ -40583,7 +40568,7 @@
         <v>4079</v>
       </c>
       <c r="B152" s="70" t="s">
-        <v>4526</v>
+        <v>4366</v>
       </c>
       <c r="C152" s="70" t="s">
         <v>31</v>
@@ -40600,7 +40585,7 @@
         <v>4080</v>
       </c>
       <c r="B153" s="70" t="s">
-        <v>4527</v>
+        <v>4367</v>
       </c>
       <c r="C153" s="70" t="s">
         <v>89</v>
@@ -40615,7 +40600,7 @@
         <v>4081</v>
       </c>
       <c r="B154" s="70" t="s">
-        <v>4528</v>
+        <v>4368</v>
       </c>
       <c r="C154" s="70" t="s">
         <v>31</v>
@@ -40632,7 +40617,7 @@
         <v>4082</v>
       </c>
       <c r="B155" s="70" t="s">
-        <v>4529</v>
+        <v>4369</v>
       </c>
       <c r="C155" s="70" t="s">
         <v>89</v>
@@ -40647,7 +40632,7 @@
         <v>4083</v>
       </c>
       <c r="B156" s="70" t="s">
-        <v>4530</v>
+        <v>4370</v>
       </c>
       <c r="C156" s="70" t="s">
         <v>31</v>
@@ -40664,7 +40649,7 @@
         <v>4084</v>
       </c>
       <c r="B157" s="70" t="s">
-        <v>4531</v>
+        <v>4371</v>
       </c>
       <c r="C157" s="70" t="s">
         <v>89</v>
@@ -40679,7 +40664,7 @@
         <v>4085</v>
       </c>
       <c r="B158" s="70" t="s">
-        <v>4532</v>
+        <v>4372</v>
       </c>
       <c r="C158" s="70" t="s">
         <v>31</v>
@@ -40696,7 +40681,7 @@
         <v>4086</v>
       </c>
       <c r="B159" s="70" t="s">
-        <v>4533</v>
+        <v>4373</v>
       </c>
       <c r="C159" s="70" t="s">
         <v>89</v>
@@ -40711,7 +40696,7 @@
         <v>4087</v>
       </c>
       <c r="B160" s="70" t="s">
-        <v>4534</v>
+        <v>4374</v>
       </c>
       <c r="C160" s="70" t="s">
         <v>31</v>
@@ -40728,7 +40713,7 @@
         <v>4088</v>
       </c>
       <c r="B161" s="70" t="s">
-        <v>4535</v>
+        <v>4375</v>
       </c>
       <c r="C161" s="70" t="s">
         <v>89</v>
@@ -40743,7 +40728,7 @@
         <v>4089</v>
       </c>
       <c r="B162" s="70" t="s">
-        <v>4536</v>
+        <v>4376</v>
       </c>
       <c r="C162" s="70" t="s">
         <v>31</v>
@@ -40760,7 +40745,7 @@
         <v>4090</v>
       </c>
       <c r="B163" s="70" t="s">
-        <v>4537</v>
+        <v>4377</v>
       </c>
       <c r="C163" s="70" t="s">
         <v>89</v>
@@ -40775,7 +40760,7 @@
         <v>4091</v>
       </c>
       <c r="B164" s="70" t="s">
-        <v>4538</v>
+        <v>4378</v>
       </c>
       <c r="C164" s="70" t="s">
         <v>31</v>
@@ -40792,7 +40777,7 @@
         <v>4092</v>
       </c>
       <c r="B165" s="70" t="s">
-        <v>4539</v>
+        <v>4379</v>
       </c>
       <c r="C165" s="70" t="s">
         <v>89</v>
@@ -40807,7 +40792,7 @@
         <v>4093</v>
       </c>
       <c r="B166" s="70" t="s">
-        <v>4540</v>
+        <v>4380</v>
       </c>
       <c r="C166" s="70" t="s">
         <v>31</v>
@@ -40824,7 +40809,7 @@
         <v>4094</v>
       </c>
       <c r="B167" s="72" t="s">
-        <v>4541</v>
+        <v>4381</v>
       </c>
       <c r="C167" s="72" t="s">
         <v>89</v>
@@ -40839,7 +40824,7 @@
         <v>4095</v>
       </c>
       <c r="B168" s="72" t="s">
-        <v>4542</v>
+        <v>4382</v>
       </c>
       <c r="C168" s="72" t="s">
         <v>31</v>
@@ -40856,7 +40841,7 @@
         <v>4096</v>
       </c>
       <c r="B169" s="72" t="s">
-        <v>4543</v>
+        <v>4383</v>
       </c>
       <c r="C169" s="72" t="s">
         <v>89</v>
@@ -40871,7 +40856,7 @@
         <v>4097</v>
       </c>
       <c r="B170" s="72" t="s">
-        <v>4544</v>
+        <v>4384</v>
       </c>
       <c r="C170" s="72" t="s">
         <v>31</v>
@@ -40888,7 +40873,7 @@
         <v>4098</v>
       </c>
       <c r="B171" s="72" t="s">
-        <v>4545</v>
+        <v>4385</v>
       </c>
       <c r="C171" s="72" t="s">
         <v>89</v>
@@ -40903,7 +40888,7 @@
         <v>4099</v>
       </c>
       <c r="B172" s="72" t="s">
-        <v>4546</v>
+        <v>4386</v>
       </c>
       <c r="C172" s="72" t="s">
         <v>31</v>
@@ -40920,7 +40905,7 @@
         <v>4100</v>
       </c>
       <c r="B173" s="74" t="s">
-        <v>4547</v>
+        <v>4387</v>
       </c>
       <c r="C173" s="74" t="s">
         <v>89</v>
@@ -40935,7 +40920,7 @@
         <v>4101</v>
       </c>
       <c r="B174" s="74" t="s">
-        <v>4548</v>
+        <v>4388</v>
       </c>
       <c r="C174" s="74" t="s">
         <v>31</v>
@@ -40952,7 +40937,7 @@
         <v>4102</v>
       </c>
       <c r="B175" s="76" t="s">
-        <v>4549</v>
+        <v>4389</v>
       </c>
       <c r="C175" s="142" t="s">
         <v>89</v>
@@ -40967,7 +40952,7 @@
         <v>4103</v>
       </c>
       <c r="B176" s="76" t="s">
-        <v>4550</v>
+        <v>4390</v>
       </c>
       <c r="C176" s="142" t="s">
         <v>31</v>
@@ -40984,7 +40969,7 @@
         <v>4104</v>
       </c>
       <c r="B177" s="76" t="s">
-        <v>4551</v>
+        <v>4391</v>
       </c>
       <c r="C177" s="142" t="s">
         <v>89</v>
@@ -40999,7 +40984,7 @@
         <v>4105</v>
       </c>
       <c r="B178" s="76" t="s">
-        <v>4552</v>
+        <v>4392</v>
       </c>
       <c r="C178" s="142" t="s">
         <v>31</v>
@@ -41016,7 +41001,7 @@
         <v>4106</v>
       </c>
       <c r="B179" s="76" t="s">
-        <v>4553</v>
+        <v>4393</v>
       </c>
       <c r="C179" s="142" t="s">
         <v>89</v>
@@ -41031,7 +41016,7 @@
         <v>4107</v>
       </c>
       <c r="B180" s="76" t="s">
-        <v>4554</v>
+        <v>4394</v>
       </c>
       <c r="C180" s="142" t="s">
         <v>31</v>
@@ -49182,7 +49167,7 @@
         <v>2962</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>4413</v>
+        <v>4317</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>89</v>
@@ -49197,7 +49182,7 @@
         <v>2971</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>4414</v>
+        <v>4318</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>31</v>
@@ -50877,7 +50862,7 @@
         <v>669</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>4556</v>
+        <v>4396</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -50909,7 +50894,7 @@
         <v>673</v>
       </c>
       <c r="B123" s="28" t="s">
-        <v>4557</v>
+        <v>4397</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -53089,7 +53074,7 @@
         <v>3138</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>4210</v>
+        <v>4449</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>31</v>
@@ -53104,7 +53089,7 @@
         <v>3139</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>4211</v>
+        <v>4406</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>31</v>
@@ -53119,7 +53104,7 @@
         <v>3140</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>4212</v>
+        <v>4407</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>89</v>
@@ -53134,7 +53119,7 @@
         <v>3141</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>4213</v>
+        <v>4408</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>31</v>
@@ -53151,7 +53136,7 @@
         <v>3142</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>4413</v>
+        <v>4317</v>
       </c>
       <c r="C11" s="52" t="s">
         <v>89</v>
@@ -53166,7 +53151,7 @@
         <v>3143</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>4414</v>
+        <v>4318</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>31</v>
@@ -53183,7 +53168,7 @@
         <v>3144</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>4214</v>
+        <v>4409</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>37</v>
@@ -53198,7 +53183,7 @@
         <v>3145</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>4215</v>
+        <v>4410</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>37</v>
@@ -53213,7 +53198,7 @@
         <v>3146</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>4216</v>
+        <v>4411</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>37</v>
@@ -53228,7 +53213,7 @@
         <v>3147</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>4217</v>
+        <v>4412</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>47</v>
@@ -53243,7 +53228,7 @@
         <v>3148</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>4218</v>
+        <v>4413</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>47</v>
@@ -53258,7 +53243,7 @@
         <v>3149</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>4220</v>
+        <v>4497</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>37</v>
@@ -53273,7 +53258,7 @@
         <v>3150</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>4219</v>
+        <v>4414</v>
       </c>
       <c r="C19" s="52" t="s">
         <v>47</v>
@@ -53288,7 +53273,7 @@
         <v>3151</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>4221</v>
+        <v>4415</v>
       </c>
       <c r="C20" s="122" t="s">
         <v>197</v>
@@ -53303,7 +53288,7 @@
         <v>3152</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>4222</v>
+        <v>4416</v>
       </c>
       <c r="C21" s="122" t="s">
         <v>201</v>
@@ -53320,7 +53305,7 @@
         <v>3153</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>4223</v>
+        <v>4417</v>
       </c>
       <c r="C22" s="122" t="s">
         <v>197</v>
@@ -53335,7 +53320,7 @@
         <v>3154</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>4224</v>
+        <v>4418</v>
       </c>
       <c r="C23" s="122" t="s">
         <v>201</v>
@@ -53352,7 +53337,7 @@
         <v>3155</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>4225</v>
+        <v>4419</v>
       </c>
       <c r="C24" s="122" t="s">
         <v>197</v>
@@ -53367,7 +53352,7 @@
         <v>3156</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>4226</v>
+        <v>4420</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>201</v>
@@ -53384,7 +53369,7 @@
         <v>3157</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>4227</v>
+        <v>4421</v>
       </c>
       <c r="C26" s="122" t="s">
         <v>197</v>
@@ -53399,7 +53384,7 @@
         <v>3158</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>4228</v>
+        <v>4422</v>
       </c>
       <c r="C27" s="122" t="s">
         <v>201</v>
@@ -53416,7 +53401,7 @@
         <v>3159</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>4229</v>
+        <v>4423</v>
       </c>
       <c r="C28" s="122" t="s">
         <v>197</v>
@@ -53431,7 +53416,7 @@
         <v>3160</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>4230</v>
+        <v>4424</v>
       </c>
       <c r="C29" s="122" t="s">
         <v>201</v>
@@ -53448,7 +53433,7 @@
         <v>3161</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>4231</v>
+        <v>4425</v>
       </c>
       <c r="C30" s="122" t="s">
         <v>197</v>
@@ -53463,7 +53448,7 @@
         <v>3162</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>4232</v>
+        <v>4426</v>
       </c>
       <c r="C31" s="122" t="s">
         <v>201</v>
@@ -53480,7 +53465,7 @@
         <v>3163</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>4233</v>
+        <v>4427</v>
       </c>
       <c r="C32" s="122" t="s">
         <v>197</v>
@@ -53495,7 +53480,7 @@
         <v>3164</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>4234</v>
+        <v>670</v>
       </c>
       <c r="C33" s="122" t="s">
         <v>201</v>
@@ -53512,7 +53497,7 @@
         <v>3165</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>4235</v>
+        <v>4428</v>
       </c>
       <c r="C34" s="123" t="s">
         <v>201</v>
@@ -53527,7 +53512,7 @@
         <v>3166</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>4236</v>
+        <v>4429</v>
       </c>
       <c r="C35" s="123" t="s">
         <v>201</v>
@@ -53542,7 +53527,7 @@
         <v>3167</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>4237</v>
+        <v>4430</v>
       </c>
       <c r="C36" s="123" t="s">
         <v>201</v>
@@ -53557,7 +53542,7 @@
         <v>3168</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>4238</v>
+        <v>4431</v>
       </c>
       <c r="C37" s="123" t="s">
         <v>201</v>
@@ -53572,7 +53557,7 @@
         <v>3169</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>4239</v>
+        <v>4432</v>
       </c>
       <c r="C38" s="123" t="s">
         <v>201</v>
@@ -53587,7 +53572,7 @@
         <v>3170</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>4240</v>
+        <v>4433</v>
       </c>
       <c r="C39" s="123" t="s">
         <v>201</v>
@@ -53602,7 +53587,7 @@
         <v>3171</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>4241</v>
+        <v>4434</v>
       </c>
       <c r="C40" s="123" t="s">
         <v>201</v>
@@ -54624,7 +54609,7 @@
         <v>3235</v>
       </c>
       <c r="B104" s="28" t="s">
-        <v>670</v>
+        <v>4396</v>
       </c>
       <c r="C104" s="130" t="s">
         <v>201</v>
@@ -55287,7 +55272,7 @@
         <v>3278</v>
       </c>
       <c r="B147" s="19" t="s">
-        <v>4242</v>
+        <v>4210</v>
       </c>
       <c r="C147" s="70" t="s">
         <v>89</v>
@@ -55302,7 +55287,7 @@
         <v>3279</v>
       </c>
       <c r="B148" s="19" t="s">
-        <v>4243</v>
+        <v>4211</v>
       </c>
       <c r="C148" s="70" t="s">
         <v>31</v>
@@ -55319,7 +55304,7 @@
         <v>3280</v>
       </c>
       <c r="B149" s="19" t="s">
-        <v>4244</v>
+        <v>4212</v>
       </c>
       <c r="C149" s="70" t="s">
         <v>89</v>
@@ -55334,7 +55319,7 @@
         <v>3281</v>
       </c>
       <c r="B150" s="19" t="s">
-        <v>4245</v>
+        <v>4213</v>
       </c>
       <c r="C150" s="70" t="s">
         <v>31</v>
@@ -55351,7 +55336,7 @@
         <v>3282</v>
       </c>
       <c r="B151" s="19" t="s">
-        <v>4246</v>
+        <v>4214</v>
       </c>
       <c r="C151" s="70" t="s">
         <v>89</v>
@@ -55366,7 +55351,7 @@
         <v>3283</v>
       </c>
       <c r="B152" s="19" t="s">
-        <v>4247</v>
+        <v>4215</v>
       </c>
       <c r="C152" s="70" t="s">
         <v>31</v>
@@ -55383,7 +55368,7 @@
         <v>3284</v>
       </c>
       <c r="B153" s="19" t="s">
-        <v>4248</v>
+        <v>4216</v>
       </c>
       <c r="C153" s="70" t="s">
         <v>89</v>
@@ -55398,7 +55383,7 @@
         <v>3285</v>
       </c>
       <c r="B154" s="19" t="s">
-        <v>4249</v>
+        <v>4217</v>
       </c>
       <c r="C154" s="70" t="s">
         <v>31</v>
@@ -55415,7 +55400,7 @@
         <v>3286</v>
       </c>
       <c r="B155" s="19" t="s">
-        <v>4250</v>
+        <v>4218</v>
       </c>
       <c r="C155" s="70" t="s">
         <v>89</v>
@@ -55430,7 +55415,7 @@
         <v>3287</v>
       </c>
       <c r="B156" s="19" t="s">
-        <v>4251</v>
+        <v>4219</v>
       </c>
       <c r="C156" s="70" t="s">
         <v>31</v>
@@ -55447,7 +55432,7 @@
         <v>3288</v>
       </c>
       <c r="B157" s="19" t="s">
-        <v>4252</v>
+        <v>4220</v>
       </c>
       <c r="C157" s="70" t="s">
         <v>89</v>
@@ -55462,7 +55447,7 @@
         <v>3289</v>
       </c>
       <c r="B158" s="19" t="s">
-        <v>4253</v>
+        <v>4221</v>
       </c>
       <c r="C158" s="70" t="s">
         <v>31</v>
@@ -55479,7 +55464,7 @@
         <v>3290</v>
       </c>
       <c r="B159" s="19" t="s">
-        <v>4254</v>
+        <v>4222</v>
       </c>
       <c r="C159" s="70" t="s">
         <v>89</v>
@@ -55494,7 +55479,7 @@
         <v>3291</v>
       </c>
       <c r="B160" s="19" t="s">
-        <v>4255</v>
+        <v>4223</v>
       </c>
       <c r="C160" s="70" t="s">
         <v>31</v>
@@ -55511,7 +55496,7 @@
         <v>3292</v>
       </c>
       <c r="B161" s="19" t="s">
-        <v>4256</v>
+        <v>4224</v>
       </c>
       <c r="C161" s="70" t="s">
         <v>89</v>
@@ -55526,7 +55511,7 @@
         <v>3293</v>
       </c>
       <c r="B162" s="19" t="s">
-        <v>4257</v>
+        <v>4225</v>
       </c>
       <c r="C162" s="70" t="s">
         <v>31</v>
@@ -55543,7 +55528,7 @@
         <v>3294</v>
       </c>
       <c r="B163" s="19" t="s">
-        <v>4258</v>
+        <v>4226</v>
       </c>
       <c r="C163" s="70" t="s">
         <v>89</v>
@@ -55558,7 +55543,7 @@
         <v>3295</v>
       </c>
       <c r="B164" s="19" t="s">
-        <v>4259</v>
+        <v>4227</v>
       </c>
       <c r="C164" s="70" t="s">
         <v>31</v>
@@ -55575,7 +55560,7 @@
         <v>3296</v>
       </c>
       <c r="B165" s="19" t="s">
-        <v>4260</v>
+        <v>4228</v>
       </c>
       <c r="C165" s="70" t="s">
         <v>89</v>
@@ -55590,7 +55575,7 @@
         <v>3297</v>
       </c>
       <c r="B166" s="19" t="s">
-        <v>4261</v>
+        <v>4229</v>
       </c>
       <c r="C166" s="70" t="s">
         <v>31</v>
@@ -55607,7 +55592,7 @@
         <v>3298</v>
       </c>
       <c r="B167" s="19" t="s">
-        <v>4262</v>
+        <v>4230</v>
       </c>
       <c r="C167" s="70" t="s">
         <v>89</v>
@@ -55622,7 +55607,7 @@
         <v>3299</v>
       </c>
       <c r="B168" s="19" t="s">
-        <v>4263</v>
+        <v>4231</v>
       </c>
       <c r="C168" s="70" t="s">
         <v>31</v>
@@ -55639,7 +55624,7 @@
         <v>3300</v>
       </c>
       <c r="B169" s="20" t="s">
-        <v>4264</v>
+        <v>4232</v>
       </c>
       <c r="C169" s="72" t="s">
         <v>89</v>
@@ -55654,7 +55639,7 @@
         <v>3301</v>
       </c>
       <c r="B170" s="20" t="s">
-        <v>4265</v>
+        <v>4233</v>
       </c>
       <c r="C170" s="72" t="s">
         <v>31</v>
@@ -55671,7 +55656,7 @@
         <v>3302</v>
       </c>
       <c r="B171" s="20" t="s">
-        <v>4266</v>
+        <v>4234</v>
       </c>
       <c r="C171" s="72" t="s">
         <v>89</v>
@@ -55686,7 +55671,7 @@
         <v>3303</v>
       </c>
       <c r="B172" s="20" t="s">
-        <v>4267</v>
+        <v>4235</v>
       </c>
       <c r="C172" s="72" t="s">
         <v>31</v>
@@ -55703,7 +55688,7 @@
         <v>3304</v>
       </c>
       <c r="B173" s="20" t="s">
-        <v>4268</v>
+        <v>4236</v>
       </c>
       <c r="C173" s="72" t="s">
         <v>89</v>
@@ -55718,7 +55703,7 @@
         <v>3305</v>
       </c>
       <c r="B174" s="20" t="s">
-        <v>4269</v>
+        <v>4237</v>
       </c>
       <c r="C174" s="72" t="s">
         <v>31</v>
@@ -55735,7 +55720,7 @@
         <v>3306</v>
       </c>
       <c r="B175" s="21" t="s">
-        <v>4270</v>
+        <v>4238</v>
       </c>
       <c r="C175" s="74" t="s">
         <v>89</v>
@@ -55750,7 +55735,7 @@
         <v>3307</v>
       </c>
       <c r="B176" s="21" t="s">
-        <v>4271</v>
+        <v>4239</v>
       </c>
       <c r="C176" s="74" t="s">
         <v>31</v>
@@ -55767,7 +55752,7 @@
         <v>3308</v>
       </c>
       <c r="B177" s="22" t="s">
-        <v>4272</v>
+        <v>4240</v>
       </c>
       <c r="C177" s="142" t="s">
         <v>89</v>
@@ -55782,7 +55767,7 @@
         <v>3309</v>
       </c>
       <c r="B178" s="22" t="s">
-        <v>4273</v>
+        <v>4241</v>
       </c>
       <c r="C178" s="142" t="s">
         <v>31</v>
@@ -55799,7 +55784,7 @@
         <v>3310</v>
       </c>
       <c r="B179" s="22" t="s">
-        <v>4274</v>
+        <v>4242</v>
       </c>
       <c r="C179" s="142" t="s">
         <v>89</v>
@@ -55814,7 +55799,7 @@
         <v>3311</v>
       </c>
       <c r="B180" s="22" t="s">
-        <v>4275</v>
+        <v>4243</v>
       </c>
       <c r="C180" s="142" t="s">
         <v>31</v>
@@ -55831,7 +55816,7 @@
         <v>3312</v>
       </c>
       <c r="B181" s="22" t="s">
-        <v>4276</v>
+        <v>4244</v>
       </c>
       <c r="C181" s="142" t="s">
         <v>89</v>
@@ -55846,7 +55831,7 @@
         <v>3313</v>
       </c>
       <c r="B182" s="22" t="s">
-        <v>4277</v>
+        <v>4245</v>
       </c>
       <c r="C182" s="142" t="s">
         <v>31</v>
@@ -56867,7 +56852,7 @@
         <v>2972</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>4415</v>
+        <v>4319</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>89</v>
@@ -56882,7 +56867,7 @@
         <v>2973</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>4416</v>
+        <v>4320</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>31</v>
@@ -58562,7 +58547,7 @@
         <v>1158</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>4559</v>
+        <v>4399</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -58594,7 +58579,7 @@
         <v>1162</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>4558</v>
+        <v>4398</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -59492,7 +59477,7 @@
         <v>1278</v>
       </c>
       <c r="B181" s="70" t="s">
-        <v>4555</v>
+        <v>4395</v>
       </c>
       <c r="C181" s="70" t="s">
         <v>31</v>
@@ -60682,26 +60667,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="059b9c67-646b-4b4e-9ab1-2b1c805d0390">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD6200282E8E804DB7E47654D11346C2" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="334b3f607926cb22599f187b4c015ce1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="059b9c67-646b-4b4e-9ab1-2b1c805d0390" xmlns:ns3="c05e7bd6-26a7-41a1-805c-893279a3732f" xmlns:ns4="6c854b04-c9c6-4391-adbe-2e73191270e7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fe548b9ff7492f3109b4e0b4a8efc8f" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="059b9c67-646b-4b4e-9ab1-2b1c805d0390"/>
@@ -60961,26 +60926,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCA6965B-A23A-4F60-9CAE-00FD555BD4D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="059b9c67-646b-4b4e-9ab1-2b1c805d0390">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A2EA77E-CA9B-4563-9A5E-2F50B3C8BA13}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c854b04-c9c6-4391-adbe-2e73191270e7"/>
-    <ds:schemaRef ds:uri="059b9c67-646b-4b4e-9ab1-2b1c805d0390"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FE51207-01AF-400E-9D05-58F426138751}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60998,4 +60964,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A2EA77E-CA9B-4563-9A5E-2F50B3C8BA13}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c854b04-c9c6-4391-adbe-2e73191270e7"/>
+    <ds:schemaRef ds:uri="059b9c67-646b-4b4e-9ab1-2b1c805d0390"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCA6965B-A23A-4F60-9CAE-00FD555BD4D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>